<commit_message>
added a new schedule to test
</commit_message>
<xml_diff>
--- a/software/conformance_test_schedule_main.xlsx
+++ b/software/conformance_test_schedule_main.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pwrgra09-admin\Documents\myPythonFiles\Root\conformance_testing_team\software\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{25C719E7-548A-4C01-9B43-2676449B12AF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D33C12C4-333F-4CD7-8590-3132D55C2F65}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38280" yWindow="-120" windowWidth="25440" windowHeight="15270" xr2:uid="{C8C0DF4B-6D5B-4BD3-847D-4558E3821A3D}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="15720" xr2:uid="{C8C0DF4B-6D5B-4BD3-847D-4558E3821A3D}"/>
   </bookViews>
   <sheets>
     <sheet name="conformance_test_schedule_main" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="35">
   <si>
     <t>enabled</t>
   </si>
@@ -137,6 +137,9 @@
   </si>
   <si>
     <t>Grid emergency event</t>
+  </si>
+  <si>
+    <t>Attemp Advanced Load up</t>
   </si>
 </sst>
 </file>
@@ -1018,17 +1021,18 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10" bestFit="1" customWidth="1"/>
-    <col min="2" max="3" width="15.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="19.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15.42578125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="9.28515625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="11.140625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="14.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="18" customWidth="1"/>
     <col min="7" max="7" width="24.85546875" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="15.42578125" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="15.140625" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="26.5703125" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="17" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="19.140625" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="19.85546875" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="24" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="18.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1084,7 +1088,7 @@
       <c r="C2" s="3">
         <v>0</v>
       </c>
-      <c r="D2" t="s">
+      <c r="D2" s="4" t="s">
         <v>12</v>
       </c>
       <c r="E2" t="str">
@@ -1120,7 +1124,7 @@
       <c r="C3" s="3">
         <v>4.8611111111111112E-3</v>
       </c>
-      <c r="D3" t="s">
+      <c r="D3" s="4" t="s">
         <v>20</v>
       </c>
       <c r="E3" t="str">
@@ -1156,7 +1160,7 @@
       <c r="C4" s="3">
         <v>8.3333333333333332E-3</v>
       </c>
-      <c r="D4" t="s">
+      <c r="D4" s="4" t="s">
         <v>16</v>
       </c>
       <c r="E4" t="str">
@@ -1192,7 +1196,7 @@
       <c r="C5" s="3">
         <v>1.5277777777777777E-2</v>
       </c>
-      <c r="D5" t="s">
+      <c r="D5" s="4" t="s">
         <v>20</v>
       </c>
       <c r="E5" t="str">
@@ -1228,7 +1232,7 @@
       <c r="C6" s="3">
         <v>1.7361111111111112E-2</v>
       </c>
-      <c r="D6" t="s">
+      <c r="D6" s="4" t="s">
         <v>16</v>
       </c>
       <c r="E6" t="str">
@@ -1264,7 +1268,7 @@
       <c r="C7" s="3">
         <v>2.4305555555555556E-2</v>
       </c>
-      <c r="D7" t="s">
+      <c r="D7" s="4" t="s">
         <v>20</v>
       </c>
       <c r="E7" t="str">
@@ -1300,7 +1304,7 @@
       <c r="C8" s="3">
         <v>2.5694444444444443E-2</v>
       </c>
-      <c r="D8" t="s">
+      <c r="D8" s="4" t="s">
         <v>16</v>
       </c>
       <c r="E8" t="str">
@@ -1336,7 +1340,7 @@
       <c r="C9" s="3">
         <v>3.2638888888888891E-2</v>
       </c>
-      <c r="D9" t="s">
+      <c r="D9" s="4" t="s">
         <v>20</v>
       </c>
       <c r="E9" t="str">
@@ -1367,69 +1371,93 @@
       </c>
       <c r="B10" t="str">
         <f>IF(F10="","",IF(F10="end","test_end",F10&amp;"_"&amp;COUNTIF($F$2:F10,F10)))</f>
-        <v>test_end</v>
+        <v>advanced_load_up_1</v>
       </c>
       <c r="C10" s="3">
-        <v>3.6111111111111108E-2</v>
-      </c>
-      <c r="D10" t="s">
+        <v>3.4027777777777775E-2</v>
+      </c>
+      <c r="D10" s="4" t="s">
         <v>20</v>
       </c>
       <c r="E10" t="str">
         <f t="shared" si="0"/>
-        <v>test</v>
+        <v>cta</v>
       </c>
       <c r="F10" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="G10" s="4"/>
+        <v>25</v>
+      </c>
+      <c r="G10" s="4" t="s">
+        <v>18</v>
+      </c>
       <c r="H10" s="4"/>
       <c r="I10" s="4"/>
       <c r="J10" s="2" t="str">
         <f>IFERROR(_xlfn.XLOOKUP(F10,'CTA Actions'!$A$2:$A$7,'CTA Actions'!$B$2:$B$7),"")</f>
-        <v/>
+        <v>3|6</v>
       </c>
       <c r="K10" s="4"/>
       <c r="L10" s="4"/>
       <c r="M10" s="4" t="s">
-        <v>22</v>
+        <v>34</v>
       </c>
     </row>
     <row r="11" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A11" s="4"/>
+      <c r="A11" s="4" t="b">
+        <v>1</v>
+      </c>
       <c r="B11" t="str">
         <f>IF(F11="","",IF(F11="end","test_end",F11&amp;"_"&amp;COUNTIF($F$2:F11,F11)))</f>
-        <v/>
-      </c>
-      <c r="C11" s="3"/>
+        <v>run_normal_5</v>
+      </c>
+      <c r="C11" s="3">
+        <v>3.5416666666666666E-2</v>
+      </c>
+      <c r="D11" s="4" t="s">
+        <v>20</v>
+      </c>
       <c r="E11" t="str">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="F11" s="4"/>
-      <c r="G11" s="4"/>
+        <v>cta</v>
+      </c>
+      <c r="F11" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="G11" s="4" t="s">
+        <v>18</v>
+      </c>
       <c r="H11" s="4"/>
       <c r="I11" s="4"/>
       <c r="J11" s="2" t="str">
         <f>IFERROR(_xlfn.XLOOKUP(F11,'CTA Actions'!$A$2:$A$7,'CTA Actions'!$B$2:$B$7),"")</f>
-        <v/>
+        <v>1|0</v>
       </c>
       <c r="K11" s="4"/>
       <c r="L11" s="4"/>
-      <c r="M11" s="4"/>
+      <c r="M11" s="4" t="s">
+        <v>19</v>
+      </c>
     </row>
     <row r="12" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A12" s="4"/>
+      <c r="A12" s="4" t="b">
+        <v>1</v>
+      </c>
       <c r="B12" t="str">
         <f>IF(F12="","",IF(F12="end","test_end",F12&amp;"_"&amp;COUNTIF($F$2:F12,F12)))</f>
-        <v/>
-      </c>
-      <c r="C12" s="3"/>
+        <v>test_end</v>
+      </c>
+      <c r="C12" s="3">
+        <v>3.6805555555555557E-2</v>
+      </c>
+      <c r="D12" s="4" t="s">
+        <v>20</v>
+      </c>
       <c r="E12" t="str">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="F12" s="4"/>
+        <v>test</v>
+      </c>
+      <c r="F12" s="4" t="s">
+        <v>21</v>
+      </c>
       <c r="G12" s="4"/>
       <c r="H12" s="4"/>
       <c r="I12" s="4"/>
@@ -1439,7 +1467,9 @@
       </c>
       <c r="K12" s="4"/>
       <c r="L12" s="4"/>
-      <c r="M12" s="4"/>
+      <c r="M12" s="4" t="s">
+        <v>22</v>
+      </c>
     </row>
     <row r="13" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A13" s="4"/>
@@ -1448,6 +1478,7 @@
         <v/>
       </c>
       <c r="C13" s="3"/>
+      <c r="D13" s="4"/>
       <c r="E13" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -1471,6 +1502,7 @@
         <v/>
       </c>
       <c r="C14" s="3"/>
+      <c r="D14" s="4"/>
       <c r="E14" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -1494,6 +1526,7 @@
         <v/>
       </c>
       <c r="C15" s="3"/>
+      <c r="D15" s="4"/>
       <c r="E15" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -1517,6 +1550,7 @@
         <v/>
       </c>
       <c r="C16" s="3"/>
+      <c r="D16" s="4"/>
       <c r="E16" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -1540,6 +1574,7 @@
         <v/>
       </c>
       <c r="C17" s="3"/>
+      <c r="D17" s="4"/>
       <c r="E17" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -1563,6 +1598,7 @@
         <v/>
       </c>
       <c r="C18" s="3"/>
+      <c r="D18" s="4"/>
       <c r="E18" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -1586,6 +1622,7 @@
         <v/>
       </c>
       <c r="C19" s="3"/>
+      <c r="D19" s="4"/>
       <c r="E19" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -1609,6 +1646,7 @@
         <v/>
       </c>
       <c r="C20" s="3"/>
+      <c r="D20" s="4"/>
       <c r="E20" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -1632,6 +1670,7 @@
         <v/>
       </c>
       <c r="C21" s="3"/>
+      <c r="D21" s="4"/>
       <c r="E21" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -1655,6 +1694,7 @@
         <v/>
       </c>
       <c r="C22" s="3"/>
+      <c r="D22" s="4"/>
       <c r="E22" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -1678,6 +1718,7 @@
         <v/>
       </c>
       <c r="C23" s="3"/>
+      <c r="D23" s="4"/>
       <c r="E23" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -1701,6 +1742,7 @@
         <v/>
       </c>
       <c r="C24" s="3"/>
+      <c r="D24" s="4"/>
       <c r="E24" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -1724,6 +1766,7 @@
         <v/>
       </c>
       <c r="C25" s="3"/>
+      <c r="D25" s="4"/>
       <c r="E25" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -1747,6 +1790,7 @@
         <v/>
       </c>
       <c r="C26" s="3"/>
+      <c r="D26" s="4"/>
       <c r="E26" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -1770,6 +1814,7 @@
         <v/>
       </c>
       <c r="C27" s="3"/>
+      <c r="D27" s="4"/>
       <c r="E27" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -1793,6 +1838,7 @@
         <v/>
       </c>
       <c r="C28" s="3"/>
+      <c r="D28" s="4"/>
       <c r="E28" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -1816,6 +1862,7 @@
         <v/>
       </c>
       <c r="C29" s="3"/>
+      <c r="D29" s="4"/>
       <c r="E29" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -1839,6 +1886,7 @@
         <v/>
       </c>
       <c r="C30" s="3"/>
+      <c r="D30" s="4"/>
       <c r="E30" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -1862,6 +1910,7 @@
         <v/>
       </c>
       <c r="C31" s="3"/>
+      <c r="D31" s="4"/>
       <c r="E31" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -1885,6 +1934,7 @@
         <v/>
       </c>
       <c r="C32" s="3"/>
+      <c r="D32" s="4"/>
       <c r="E32" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -1908,6 +1958,7 @@
         <v/>
       </c>
       <c r="C33" s="3"/>
+      <c r="D33" s="4"/>
       <c r="E33" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -1931,6 +1982,7 @@
         <v/>
       </c>
       <c r="C34" s="3"/>
+      <c r="D34" s="4"/>
       <c r="E34" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -1954,6 +2006,7 @@
         <v/>
       </c>
       <c r="C35" s="3"/>
+      <c r="D35" s="4"/>
       <c r="E35" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -1977,6 +2030,7 @@
         <v/>
       </c>
       <c r="C36" s="3"/>
+      <c r="D36" s="4"/>
       <c r="E36" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -2000,6 +2054,7 @@
         <v/>
       </c>
       <c r="C37" s="3"/>
+      <c r="D37" s="4"/>
       <c r="E37" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -2023,6 +2078,7 @@
         <v/>
       </c>
       <c r="C38" s="3"/>
+      <c r="D38" s="4"/>
       <c r="E38" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -2046,6 +2102,7 @@
         <v/>
       </c>
       <c r="C39" s="3"/>
+      <c r="D39" s="4"/>
       <c r="E39" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -2069,6 +2126,7 @@
         <v/>
       </c>
       <c r="C40" s="3"/>
+      <c r="D40" s="4"/>
       <c r="E40" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -2092,6 +2150,7 @@
         <v/>
       </c>
       <c r="C41" s="3"/>
+      <c r="D41" s="4"/>
       <c r="E41" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -2115,6 +2174,7 @@
         <v/>
       </c>
       <c r="C42" s="3"/>
+      <c r="D42" s="4"/>
       <c r="E42" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -2138,6 +2198,7 @@
         <v/>
       </c>
       <c r="C43" s="3"/>
+      <c r="D43" s="4"/>
       <c r="E43" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -2161,6 +2222,7 @@
         <v/>
       </c>
       <c r="C44" s="3"/>
+      <c r="D44" s="4"/>
       <c r="E44" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -2184,6 +2246,7 @@
         <v/>
       </c>
       <c r="C45" s="3"/>
+      <c r="D45" s="4"/>
       <c r="E45" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -2207,6 +2270,7 @@
         <v/>
       </c>
       <c r="C46" s="3"/>
+      <c r="D46" s="4"/>
       <c r="E46" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -2230,6 +2294,7 @@
         <v/>
       </c>
       <c r="C47" s="3"/>
+      <c r="D47" s="4"/>
       <c r="E47" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -2253,6 +2318,7 @@
         <v/>
       </c>
       <c r="C48" s="3"/>
+      <c r="D48" s="4"/>
       <c r="E48" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -2276,6 +2342,7 @@
         <v/>
       </c>
       <c r="C49" s="3"/>
+      <c r="D49" s="4"/>
       <c r="E49" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -2299,6 +2366,7 @@
         <v/>
       </c>
       <c r="C50" s="3"/>
+      <c r="D50" s="4"/>
       <c r="E50" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -2322,6 +2390,7 @@
         <v/>
       </c>
       <c r="C51" s="3"/>
+      <c r="D51" s="4"/>
       <c r="E51" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -2345,6 +2414,7 @@
         <v/>
       </c>
       <c r="C52" s="3"/>
+      <c r="D52" s="4"/>
       <c r="E52" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -2368,6 +2438,7 @@
         <v/>
       </c>
       <c r="C53" s="3"/>
+      <c r="D53" s="4"/>
       <c r="E53" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -2391,6 +2462,7 @@
         <v/>
       </c>
       <c r="C54" s="3"/>
+      <c r="D54" s="4"/>
       <c r="E54" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -2414,6 +2486,7 @@
         <v/>
       </c>
       <c r="C55" s="3"/>
+      <c r="D55" s="4"/>
       <c r="E55" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -2437,6 +2510,7 @@
         <v/>
       </c>
       <c r="C56" s="3"/>
+      <c r="D56" s="4"/>
       <c r="E56" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -2460,6 +2534,7 @@
         <v/>
       </c>
       <c r="C57" s="3"/>
+      <c r="D57" s="4"/>
       <c r="E57" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -2483,6 +2558,7 @@
         <v/>
       </c>
       <c r="C58" s="3"/>
+      <c r="D58" s="4"/>
       <c r="E58" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -2506,6 +2582,7 @@
         <v/>
       </c>
       <c r="C59" s="3"/>
+      <c r="D59" s="4"/>
       <c r="E59" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -2529,6 +2606,7 @@
         <v/>
       </c>
       <c r="C60" s="3"/>
+      <c r="D60" s="4"/>
       <c r="E60" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -2552,6 +2630,7 @@
         <v/>
       </c>
       <c r="C61" s="3"/>
+      <c r="D61" s="4"/>
       <c r="E61" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -2575,6 +2654,7 @@
         <v/>
       </c>
       <c r="C62" s="3"/>
+      <c r="D62" s="4"/>
       <c r="E62" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -2598,6 +2678,7 @@
         <v/>
       </c>
       <c r="C63" s="3"/>
+      <c r="D63" s="4"/>
       <c r="E63" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -2621,6 +2702,7 @@
         <v/>
       </c>
       <c r="C64" s="3"/>
+      <c r="D64" s="4"/>
       <c r="E64" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -2644,6 +2726,7 @@
         <v/>
       </c>
       <c r="C65" s="3"/>
+      <c r="D65" s="4"/>
       <c r="E65" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -2667,6 +2750,7 @@
         <v/>
       </c>
       <c r="C66" s="3"/>
+      <c r="D66" s="4"/>
       <c r="E66" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -2690,6 +2774,7 @@
         <v/>
       </c>
       <c r="C67" s="3"/>
+      <c r="D67" s="4"/>
       <c r="E67" t="str">
         <f t="shared" ref="E67:E130" si="1">IF(F67="","",IF(F67="water_draw","water_draw",IF(F67="end","test","cta")))</f>
         <v/>
@@ -2713,6 +2798,7 @@
         <v/>
       </c>
       <c r="C68" s="3"/>
+      <c r="D68" s="4"/>
       <c r="E68" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -2736,6 +2822,7 @@
         <v/>
       </c>
       <c r="C69" s="3"/>
+      <c r="D69" s="4"/>
       <c r="E69" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -2759,6 +2846,7 @@
         <v/>
       </c>
       <c r="C70" s="3"/>
+      <c r="D70" s="4"/>
       <c r="E70" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -2782,6 +2870,7 @@
         <v/>
       </c>
       <c r="C71" s="3"/>
+      <c r="D71" s="4"/>
       <c r="E71" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -2805,6 +2894,7 @@
         <v/>
       </c>
       <c r="C72" s="3"/>
+      <c r="D72" s="4"/>
       <c r="E72" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -2828,6 +2918,7 @@
         <v/>
       </c>
       <c r="C73" s="3"/>
+      <c r="D73" s="4"/>
       <c r="E73" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -2851,6 +2942,7 @@
         <v/>
       </c>
       <c r="C74" s="3"/>
+      <c r="D74" s="4"/>
       <c r="E74" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -2874,6 +2966,7 @@
         <v/>
       </c>
       <c r="C75" s="3"/>
+      <c r="D75" s="4"/>
       <c r="E75" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -2897,6 +2990,7 @@
         <v/>
       </c>
       <c r="C76" s="3"/>
+      <c r="D76" s="4"/>
       <c r="E76" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -2920,6 +3014,7 @@
         <v/>
       </c>
       <c r="C77" s="3"/>
+      <c r="D77" s="4"/>
       <c r="E77" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -2943,6 +3038,7 @@
         <v/>
       </c>
       <c r="C78" s="3"/>
+      <c r="D78" s="4"/>
       <c r="E78" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -2966,6 +3062,7 @@
         <v/>
       </c>
       <c r="C79" s="3"/>
+      <c r="D79" s="4"/>
       <c r="E79" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -2989,6 +3086,7 @@
         <v/>
       </c>
       <c r="C80" s="3"/>
+      <c r="D80" s="4"/>
       <c r="E80" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -3012,6 +3110,7 @@
         <v/>
       </c>
       <c r="C81" s="3"/>
+      <c r="D81" s="4"/>
       <c r="E81" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -3035,6 +3134,7 @@
         <v/>
       </c>
       <c r="C82" s="3"/>
+      <c r="D82" s="4"/>
       <c r="E82" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -3058,6 +3158,7 @@
         <v/>
       </c>
       <c r="C83" s="3"/>
+      <c r="D83" s="4"/>
       <c r="E83" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -3081,6 +3182,7 @@
         <v/>
       </c>
       <c r="C84" s="3"/>
+      <c r="D84" s="4"/>
       <c r="E84" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -3104,6 +3206,7 @@
         <v/>
       </c>
       <c r="C85" s="3"/>
+      <c r="D85" s="4"/>
       <c r="E85" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -3127,6 +3230,7 @@
         <v/>
       </c>
       <c r="C86" s="3"/>
+      <c r="D86" s="4"/>
       <c r="E86" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -3150,6 +3254,7 @@
         <v/>
       </c>
       <c r="C87" s="3"/>
+      <c r="D87" s="4"/>
       <c r="E87" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -3173,6 +3278,7 @@
         <v/>
       </c>
       <c r="C88" s="3"/>
+      <c r="D88" s="4"/>
       <c r="E88" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -3196,6 +3302,7 @@
         <v/>
       </c>
       <c r="C89" s="3"/>
+      <c r="D89" s="4"/>
       <c r="E89" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -3219,6 +3326,7 @@
         <v/>
       </c>
       <c r="C90" s="3"/>
+      <c r="D90" s="4"/>
       <c r="E90" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -3242,6 +3350,7 @@
         <v/>
       </c>
       <c r="C91" s="3"/>
+      <c r="D91" s="4"/>
       <c r="E91" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -3265,6 +3374,7 @@
         <v/>
       </c>
       <c r="C92" s="3"/>
+      <c r="D92" s="4"/>
       <c r="E92" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -3288,6 +3398,7 @@
         <v/>
       </c>
       <c r="C93" s="3"/>
+      <c r="D93" s="4"/>
       <c r="E93" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -3311,6 +3422,7 @@
         <v/>
       </c>
       <c r="C94" s="3"/>
+      <c r="D94" s="4"/>
       <c r="E94" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -3334,6 +3446,7 @@
         <v/>
       </c>
       <c r="C95" s="3"/>
+      <c r="D95" s="4"/>
       <c r="E95" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -3357,6 +3470,7 @@
         <v/>
       </c>
       <c r="C96" s="3"/>
+      <c r="D96" s="4"/>
       <c r="E96" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -3380,6 +3494,7 @@
         <v/>
       </c>
       <c r="C97" s="3"/>
+      <c r="D97" s="4"/>
       <c r="E97" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -3403,6 +3518,7 @@
         <v/>
       </c>
       <c r="C98" s="3"/>
+      <c r="D98" s="4"/>
       <c r="E98" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -3426,6 +3542,7 @@
         <v/>
       </c>
       <c r="C99" s="3"/>
+      <c r="D99" s="4"/>
       <c r="E99" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -3449,6 +3566,7 @@
         <v/>
       </c>
       <c r="C100" s="3"/>
+      <c r="D100" s="4"/>
       <c r="E100" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -3472,6 +3590,7 @@
         <v/>
       </c>
       <c r="C101" s="3"/>
+      <c r="D101" s="4"/>
       <c r="E101" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -3495,6 +3614,7 @@
         <v/>
       </c>
       <c r="C102" s="3"/>
+      <c r="D102" s="4"/>
       <c r="E102" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -3518,6 +3638,7 @@
         <v/>
       </c>
       <c r="C103" s="3"/>
+      <c r="D103" s="4"/>
       <c r="E103" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -3541,6 +3662,7 @@
         <v/>
       </c>
       <c r="C104" s="3"/>
+      <c r="D104" s="4"/>
       <c r="E104" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -3564,6 +3686,7 @@
         <v/>
       </c>
       <c r="C105" s="3"/>
+      <c r="D105" s="4"/>
       <c r="E105" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -3587,6 +3710,7 @@
         <v/>
       </c>
       <c r="C106" s="3"/>
+      <c r="D106" s="4"/>
       <c r="E106" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -3610,6 +3734,7 @@
         <v/>
       </c>
       <c r="C107" s="3"/>
+      <c r="D107" s="4"/>
       <c r="E107" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -3633,6 +3758,7 @@
         <v/>
       </c>
       <c r="C108" s="3"/>
+      <c r="D108" s="4"/>
       <c r="E108" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -3656,6 +3782,7 @@
         <v/>
       </c>
       <c r="C109" s="3"/>
+      <c r="D109" s="4"/>
       <c r="E109" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -3679,6 +3806,7 @@
         <v/>
       </c>
       <c r="C110" s="3"/>
+      <c r="D110" s="4"/>
       <c r="E110" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -3702,6 +3830,7 @@
         <v/>
       </c>
       <c r="C111" s="3"/>
+      <c r="D111" s="4"/>
       <c r="E111" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -3725,6 +3854,7 @@
         <v/>
       </c>
       <c r="C112" s="3"/>
+      <c r="D112" s="4"/>
       <c r="E112" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -3748,6 +3878,7 @@
         <v/>
       </c>
       <c r="C113" s="3"/>
+      <c r="D113" s="4"/>
       <c r="E113" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -3771,6 +3902,7 @@
         <v/>
       </c>
       <c r="C114" s="3"/>
+      <c r="D114" s="4"/>
       <c r="E114" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -3794,6 +3926,7 @@
         <v/>
       </c>
       <c r="C115" s="3"/>
+      <c r="D115" s="4"/>
       <c r="E115" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -3817,6 +3950,7 @@
         <v/>
       </c>
       <c r="C116" s="3"/>
+      <c r="D116" s="4"/>
       <c r="E116" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -3840,6 +3974,7 @@
         <v/>
       </c>
       <c r="C117" s="3"/>
+      <c r="D117" s="4"/>
       <c r="E117" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -3863,6 +3998,7 @@
         <v/>
       </c>
       <c r="C118" s="3"/>
+      <c r="D118" s="4"/>
       <c r="E118" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -3886,6 +4022,7 @@
         <v/>
       </c>
       <c r="C119" s="3"/>
+      <c r="D119" s="4"/>
       <c r="E119" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -3909,6 +4046,7 @@
         <v/>
       </c>
       <c r="C120" s="3"/>
+      <c r="D120" s="4"/>
       <c r="E120" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -3932,6 +4070,7 @@
         <v/>
       </c>
       <c r="C121" s="3"/>
+      <c r="D121" s="4"/>
       <c r="E121" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -3955,6 +4094,7 @@
         <v/>
       </c>
       <c r="C122" s="3"/>
+      <c r="D122" s="4"/>
       <c r="E122" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -3978,6 +4118,7 @@
         <v/>
       </c>
       <c r="C123" s="3"/>
+      <c r="D123" s="4"/>
       <c r="E123" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -4001,6 +4142,7 @@
         <v/>
       </c>
       <c r="C124" s="3"/>
+      <c r="D124" s="4"/>
       <c r="E124" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -4024,6 +4166,7 @@
         <v/>
       </c>
       <c r="C125" s="3"/>
+      <c r="D125" s="4"/>
       <c r="E125" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -4047,6 +4190,7 @@
         <v/>
       </c>
       <c r="C126" s="3"/>
+      <c r="D126" s="4"/>
       <c r="E126" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -4070,6 +4214,7 @@
         <v/>
       </c>
       <c r="C127" s="3"/>
+      <c r="D127" s="4"/>
       <c r="E127" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -4093,6 +4238,7 @@
         <v/>
       </c>
       <c r="C128" s="3"/>
+      <c r="D128" s="4"/>
       <c r="E128" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -4116,6 +4262,7 @@
         <v/>
       </c>
       <c r="C129" s="3"/>
+      <c r="D129" s="4"/>
       <c r="E129" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -4139,6 +4286,7 @@
         <v/>
       </c>
       <c r="C130" s="3"/>
+      <c r="D130" s="4"/>
       <c r="E130" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -4162,6 +4310,7 @@
         <v/>
       </c>
       <c r="C131" s="3"/>
+      <c r="D131" s="4"/>
       <c r="E131" t="str">
         <f t="shared" ref="E131:E194" si="2">IF(F131="","",IF(F131="water_draw","water_draw",IF(F131="end","test","cta")))</f>
         <v/>
@@ -4185,6 +4334,7 @@
         <v/>
       </c>
       <c r="C132" s="3"/>
+      <c r="D132" s="4"/>
       <c r="E132" t="str">
         <f t="shared" si="2"/>
         <v/>
@@ -4208,6 +4358,7 @@
         <v/>
       </c>
       <c r="C133" s="3"/>
+      <c r="D133" s="4"/>
       <c r="E133" t="str">
         <f t="shared" si="2"/>
         <v/>
@@ -4231,6 +4382,7 @@
         <v/>
       </c>
       <c r="C134" s="3"/>
+      <c r="D134" s="4"/>
       <c r="E134" t="str">
         <f t="shared" si="2"/>
         <v/>
@@ -4254,6 +4406,7 @@
         <v/>
       </c>
       <c r="C135" s="3"/>
+      <c r="D135" s="4"/>
       <c r="E135" t="str">
         <f t="shared" si="2"/>
         <v/>
@@ -4277,6 +4430,7 @@
         <v/>
       </c>
       <c r="C136" s="3"/>
+      <c r="D136" s="4"/>
       <c r="E136" t="str">
         <f t="shared" si="2"/>
         <v/>
@@ -4300,6 +4454,7 @@
         <v/>
       </c>
       <c r="C137" s="3"/>
+      <c r="D137" s="4"/>
       <c r="E137" t="str">
         <f t="shared" si="2"/>
         <v/>
@@ -4323,6 +4478,7 @@
         <v/>
       </c>
       <c r="C138" s="3"/>
+      <c r="D138" s="4"/>
       <c r="E138" t="str">
         <f t="shared" si="2"/>
         <v/>
@@ -4346,6 +4502,7 @@
         <v/>
       </c>
       <c r="C139" s="3"/>
+      <c r="D139" s="4"/>
       <c r="E139" t="str">
         <f t="shared" si="2"/>
         <v/>
@@ -4369,6 +4526,7 @@
         <v/>
       </c>
       <c r="C140" s="3"/>
+      <c r="D140" s="4"/>
       <c r="E140" t="str">
         <f t="shared" si="2"/>
         <v/>
@@ -4392,6 +4550,7 @@
         <v/>
       </c>
       <c r="C141" s="3"/>
+      <c r="D141" s="4"/>
       <c r="E141" t="str">
         <f t="shared" si="2"/>
         <v/>
@@ -4415,6 +4574,7 @@
         <v/>
       </c>
       <c r="C142" s="3"/>
+      <c r="D142" s="4"/>
       <c r="E142" t="str">
         <f t="shared" si="2"/>
         <v/>
@@ -4438,6 +4598,7 @@
         <v/>
       </c>
       <c r="C143" s="3"/>
+      <c r="D143" s="4"/>
       <c r="E143" t="str">
         <f t="shared" si="2"/>
         <v/>
@@ -4461,6 +4622,7 @@
         <v/>
       </c>
       <c r="C144" s="3"/>
+      <c r="D144" s="4"/>
       <c r="E144" t="str">
         <f t="shared" si="2"/>
         <v/>
@@ -4484,6 +4646,7 @@
         <v/>
       </c>
       <c r="C145" s="3"/>
+      <c r="D145" s="4"/>
       <c r="E145" t="str">
         <f t="shared" si="2"/>
         <v/>
@@ -4507,6 +4670,7 @@
         <v/>
       </c>
       <c r="C146" s="3"/>
+      <c r="D146" s="4"/>
       <c r="E146" t="str">
         <f t="shared" si="2"/>
         <v/>
@@ -4530,6 +4694,7 @@
         <v/>
       </c>
       <c r="C147" s="3"/>
+      <c r="D147" s="4"/>
       <c r="E147" t="str">
         <f t="shared" si="2"/>
         <v/>
@@ -4553,6 +4718,7 @@
         <v/>
       </c>
       <c r="C148" s="3"/>
+      <c r="D148" s="4"/>
       <c r="E148" t="str">
         <f t="shared" si="2"/>
         <v/>
@@ -4576,6 +4742,7 @@
         <v/>
       </c>
       <c r="C149" s="3"/>
+      <c r="D149" s="4"/>
       <c r="E149" t="str">
         <f t="shared" si="2"/>
         <v/>
@@ -4599,6 +4766,7 @@
         <v/>
       </c>
       <c r="C150" s="3"/>
+      <c r="D150" s="4"/>
       <c r="E150" t="str">
         <f t="shared" si="2"/>
         <v/>
@@ -4622,6 +4790,7 @@
         <v/>
       </c>
       <c r="C151" s="3"/>
+      <c r="D151" s="4"/>
       <c r="E151" t="str">
         <f t="shared" si="2"/>
         <v/>
@@ -4645,6 +4814,7 @@
         <v/>
       </c>
       <c r="C152" s="3"/>
+      <c r="D152" s="4"/>
       <c r="E152" t="str">
         <f t="shared" si="2"/>
         <v/>
@@ -4668,6 +4838,7 @@
         <v/>
       </c>
       <c r="C153" s="3"/>
+      <c r="D153" s="4"/>
       <c r="E153" t="str">
         <f t="shared" si="2"/>
         <v/>
@@ -4691,6 +4862,7 @@
         <v/>
       </c>
       <c r="C154" s="3"/>
+      <c r="D154" s="4"/>
       <c r="E154" t="str">
         <f t="shared" si="2"/>
         <v/>
@@ -4714,6 +4886,7 @@
         <v/>
       </c>
       <c r="C155" s="3"/>
+      <c r="D155" s="4"/>
       <c r="E155" t="str">
         <f t="shared" si="2"/>
         <v/>
@@ -4737,6 +4910,7 @@
         <v/>
       </c>
       <c r="C156" s="3"/>
+      <c r="D156" s="4"/>
       <c r="E156" t="str">
         <f t="shared" si="2"/>
         <v/>
@@ -4760,6 +4934,7 @@
         <v/>
       </c>
       <c r="C157" s="3"/>
+      <c r="D157" s="4"/>
       <c r="E157" t="str">
         <f t="shared" si="2"/>
         <v/>
@@ -4783,6 +4958,7 @@
         <v/>
       </c>
       <c r="C158" s="3"/>
+      <c r="D158" s="4"/>
       <c r="E158" t="str">
         <f t="shared" si="2"/>
         <v/>
@@ -4806,6 +4982,7 @@
         <v/>
       </c>
       <c r="C159" s="3"/>
+      <c r="D159" s="4"/>
       <c r="E159" t="str">
         <f t="shared" si="2"/>
         <v/>
@@ -4829,6 +5006,7 @@
         <v/>
       </c>
       <c r="C160" s="3"/>
+      <c r="D160" s="4"/>
       <c r="E160" t="str">
         <f t="shared" si="2"/>
         <v/>
@@ -4852,6 +5030,7 @@
         <v/>
       </c>
       <c r="C161" s="3"/>
+      <c r="D161" s="4"/>
       <c r="E161" t="str">
         <f t="shared" si="2"/>
         <v/>
@@ -4875,6 +5054,7 @@
         <v/>
       </c>
       <c r="C162" s="3"/>
+      <c r="D162" s="4"/>
       <c r="E162" t="str">
         <f t="shared" si="2"/>
         <v/>
@@ -4898,6 +5078,7 @@
         <v/>
       </c>
       <c r="C163" s="3"/>
+      <c r="D163" s="4"/>
       <c r="E163" t="str">
         <f t="shared" si="2"/>
         <v/>
@@ -4921,6 +5102,7 @@
         <v/>
       </c>
       <c r="C164" s="3"/>
+      <c r="D164" s="4"/>
       <c r="E164" t="str">
         <f t="shared" si="2"/>
         <v/>
@@ -4944,6 +5126,7 @@
         <v/>
       </c>
       <c r="C165" s="3"/>
+      <c r="D165" s="4"/>
       <c r="E165" t="str">
         <f t="shared" si="2"/>
         <v/>
@@ -4967,6 +5150,7 @@
         <v/>
       </c>
       <c r="C166" s="3"/>
+      <c r="D166" s="4"/>
       <c r="E166" t="str">
         <f t="shared" si="2"/>
         <v/>
@@ -4990,6 +5174,7 @@
         <v/>
       </c>
       <c r="C167" s="3"/>
+      <c r="D167" s="4"/>
       <c r="E167" t="str">
         <f t="shared" si="2"/>
         <v/>
@@ -5013,6 +5198,7 @@
         <v/>
       </c>
       <c r="C168" s="3"/>
+      <c r="D168" s="4"/>
       <c r="E168" t="str">
         <f t="shared" si="2"/>
         <v/>
@@ -5036,6 +5222,7 @@
         <v/>
       </c>
       <c r="C169" s="3"/>
+      <c r="D169" s="4"/>
       <c r="E169" t="str">
         <f t="shared" si="2"/>
         <v/>
@@ -5059,6 +5246,7 @@
         <v/>
       </c>
       <c r="C170" s="3"/>
+      <c r="D170" s="4"/>
       <c r="E170" t="str">
         <f t="shared" si="2"/>
         <v/>
@@ -5082,6 +5270,7 @@
         <v/>
       </c>
       <c r="C171" s="3"/>
+      <c r="D171" s="4"/>
       <c r="E171" t="str">
         <f t="shared" si="2"/>
         <v/>
@@ -5105,6 +5294,7 @@
         <v/>
       </c>
       <c r="C172" s="3"/>
+      <c r="D172" s="4"/>
       <c r="E172" t="str">
         <f t="shared" si="2"/>
         <v/>
@@ -5128,6 +5318,7 @@
         <v/>
       </c>
       <c r="C173" s="3"/>
+      <c r="D173" s="4"/>
       <c r="E173" t="str">
         <f t="shared" si="2"/>
         <v/>
@@ -5151,6 +5342,7 @@
         <v/>
       </c>
       <c r="C174" s="3"/>
+      <c r="D174" s="4"/>
       <c r="E174" t="str">
         <f t="shared" si="2"/>
         <v/>
@@ -5174,6 +5366,7 @@
         <v/>
       </c>
       <c r="C175" s="3"/>
+      <c r="D175" s="4"/>
       <c r="E175" t="str">
         <f t="shared" si="2"/>
         <v/>
@@ -5197,6 +5390,7 @@
         <v/>
       </c>
       <c r="C176" s="3"/>
+      <c r="D176" s="4"/>
       <c r="E176" t="str">
         <f t="shared" si="2"/>
         <v/>
@@ -5220,6 +5414,7 @@
         <v/>
       </c>
       <c r="C177" s="3"/>
+      <c r="D177" s="4"/>
       <c r="E177" t="str">
         <f t="shared" si="2"/>
         <v/>
@@ -5243,6 +5438,7 @@
         <v/>
       </c>
       <c r="C178" s="3"/>
+      <c r="D178" s="4"/>
       <c r="E178" t="str">
         <f t="shared" si="2"/>
         <v/>
@@ -5266,6 +5462,7 @@
         <v/>
       </c>
       <c r="C179" s="3"/>
+      <c r="D179" s="4"/>
       <c r="E179" t="str">
         <f t="shared" si="2"/>
         <v/>
@@ -5289,6 +5486,7 @@
         <v/>
       </c>
       <c r="C180" s="3"/>
+      <c r="D180" s="4"/>
       <c r="E180" t="str">
         <f t="shared" si="2"/>
         <v/>
@@ -5312,6 +5510,7 @@
         <v/>
       </c>
       <c r="C181" s="3"/>
+      <c r="D181" s="4"/>
       <c r="E181" t="str">
         <f t="shared" si="2"/>
         <v/>
@@ -5335,6 +5534,7 @@
         <v/>
       </c>
       <c r="C182" s="3"/>
+      <c r="D182" s="4"/>
       <c r="E182" t="str">
         <f t="shared" si="2"/>
         <v/>
@@ -5358,6 +5558,7 @@
         <v/>
       </c>
       <c r="C183" s="3"/>
+      <c r="D183" s="4"/>
       <c r="E183" t="str">
         <f t="shared" si="2"/>
         <v/>
@@ -5381,6 +5582,7 @@
         <v/>
       </c>
       <c r="C184" s="3"/>
+      <c r="D184" s="4"/>
       <c r="E184" t="str">
         <f t="shared" si="2"/>
         <v/>
@@ -5404,6 +5606,7 @@
         <v/>
       </c>
       <c r="C185" s="3"/>
+      <c r="D185" s="4"/>
       <c r="E185" t="str">
         <f t="shared" si="2"/>
         <v/>
@@ -5427,6 +5630,7 @@
         <v/>
       </c>
       <c r="C186" s="3"/>
+      <c r="D186" s="4"/>
       <c r="E186" t="str">
         <f t="shared" si="2"/>
         <v/>
@@ -5450,6 +5654,7 @@
         <v/>
       </c>
       <c r="C187" s="3"/>
+      <c r="D187" s="4"/>
       <c r="E187" t="str">
         <f t="shared" si="2"/>
         <v/>
@@ -5473,6 +5678,7 @@
         <v/>
       </c>
       <c r="C188" s="3"/>
+      <c r="D188" s="4"/>
       <c r="E188" t="str">
         <f t="shared" si="2"/>
         <v/>
@@ -5496,6 +5702,7 @@
         <v/>
       </c>
       <c r="C189" s="3"/>
+      <c r="D189" s="4"/>
       <c r="E189" t="str">
         <f t="shared" si="2"/>
         <v/>
@@ -5519,6 +5726,7 @@
         <v/>
       </c>
       <c r="C190" s="3"/>
+      <c r="D190" s="4"/>
       <c r="E190" t="str">
         <f t="shared" si="2"/>
         <v/>
@@ -5542,6 +5750,7 @@
         <v/>
       </c>
       <c r="C191" s="3"/>
+      <c r="D191" s="4"/>
       <c r="E191" t="str">
         <f t="shared" si="2"/>
         <v/>
@@ -5565,6 +5774,7 @@
         <v/>
       </c>
       <c r="C192" s="3"/>
+      <c r="D192" s="4"/>
       <c r="E192" t="str">
         <f t="shared" si="2"/>
         <v/>
@@ -5588,6 +5798,7 @@
         <v/>
       </c>
       <c r="C193" s="3"/>
+      <c r="D193" s="4"/>
       <c r="E193" t="str">
         <f t="shared" si="2"/>
         <v/>
@@ -5611,6 +5822,7 @@
         <v/>
       </c>
       <c r="C194" s="3"/>
+      <c r="D194" s="4"/>
       <c r="E194" t="str">
         <f t="shared" si="2"/>
         <v/>
@@ -5634,6 +5846,7 @@
         <v/>
       </c>
       <c r="C195" s="3"/>
+      <c r="D195" s="4"/>
       <c r="E195" t="str">
         <f t="shared" ref="E195:E258" si="3">IF(F195="","",IF(F195="water_draw","water_draw",IF(F195="end","test","cta")))</f>
         <v/>
@@ -5657,6 +5870,7 @@
         <v/>
       </c>
       <c r="C196" s="3"/>
+      <c r="D196" s="4"/>
       <c r="E196" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -5680,6 +5894,7 @@
         <v/>
       </c>
       <c r="C197" s="3"/>
+      <c r="D197" s="4"/>
       <c r="E197" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -5703,6 +5918,7 @@
         <v/>
       </c>
       <c r="C198" s="3"/>
+      <c r="D198" s="4"/>
       <c r="E198" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -5726,6 +5942,7 @@
         <v/>
       </c>
       <c r="C199" s="3"/>
+      <c r="D199" s="4"/>
       <c r="E199" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -5749,6 +5966,7 @@
         <v/>
       </c>
       <c r="C200" s="3"/>
+      <c r="D200" s="4"/>
       <c r="E200" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -5772,6 +5990,7 @@
         <v/>
       </c>
       <c r="C201" s="3"/>
+      <c r="D201" s="4"/>
       <c r="E201" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -5795,6 +6014,7 @@
         <v/>
       </c>
       <c r="C202" s="3"/>
+      <c r="D202" s="4"/>
       <c r="E202" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -5818,6 +6038,7 @@
         <v/>
       </c>
       <c r="C203" s="3"/>
+      <c r="D203" s="4"/>
       <c r="E203" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -5841,6 +6062,7 @@
         <v/>
       </c>
       <c r="C204" s="3"/>
+      <c r="D204" s="4"/>
       <c r="E204" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -5864,6 +6086,7 @@
         <v/>
       </c>
       <c r="C205" s="3"/>
+      <c r="D205" s="4"/>
       <c r="E205" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -5887,6 +6110,7 @@
         <v/>
       </c>
       <c r="C206" s="3"/>
+      <c r="D206" s="4"/>
       <c r="E206" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -5910,6 +6134,7 @@
         <v/>
       </c>
       <c r="C207" s="3"/>
+      <c r="D207" s="4"/>
       <c r="E207" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -5933,6 +6158,7 @@
         <v/>
       </c>
       <c r="C208" s="3"/>
+      <c r="D208" s="4"/>
       <c r="E208" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -5956,6 +6182,7 @@
         <v/>
       </c>
       <c r="C209" s="3"/>
+      <c r="D209" s="4"/>
       <c r="E209" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -5979,6 +6206,7 @@
         <v/>
       </c>
       <c r="C210" s="3"/>
+      <c r="D210" s="4"/>
       <c r="E210" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -6002,6 +6230,7 @@
         <v/>
       </c>
       <c r="C211" s="3"/>
+      <c r="D211" s="4"/>
       <c r="E211" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -6025,6 +6254,7 @@
         <v/>
       </c>
       <c r="C212" s="3"/>
+      <c r="D212" s="4"/>
       <c r="E212" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -6048,6 +6278,7 @@
         <v/>
       </c>
       <c r="C213" s="3"/>
+      <c r="D213" s="4"/>
       <c r="E213" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -6071,6 +6302,7 @@
         <v/>
       </c>
       <c r="C214" s="3"/>
+      <c r="D214" s="4"/>
       <c r="E214" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -6094,6 +6326,7 @@
         <v/>
       </c>
       <c r="C215" s="3"/>
+      <c r="D215" s="4"/>
       <c r="E215" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -6117,6 +6350,7 @@
         <v/>
       </c>
       <c r="C216" s="3"/>
+      <c r="D216" s="4"/>
       <c r="E216" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -6140,6 +6374,7 @@
         <v/>
       </c>
       <c r="C217" s="3"/>
+      <c r="D217" s="4"/>
       <c r="E217" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -6163,6 +6398,7 @@
         <v/>
       </c>
       <c r="C218" s="3"/>
+      <c r="D218" s="4"/>
       <c r="E218" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -6186,6 +6422,7 @@
         <v/>
       </c>
       <c r="C219" s="3"/>
+      <c r="D219" s="4"/>
       <c r="E219" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -6209,6 +6446,7 @@
         <v/>
       </c>
       <c r="C220" s="3"/>
+      <c r="D220" s="4"/>
       <c r="E220" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -6232,6 +6470,7 @@
         <v/>
       </c>
       <c r="C221" s="3"/>
+      <c r="D221" s="4"/>
       <c r="E221" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -6255,6 +6494,7 @@
         <v/>
       </c>
       <c r="C222" s="3"/>
+      <c r="D222" s="4"/>
       <c r="E222" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -6278,6 +6518,7 @@
         <v/>
       </c>
       <c r="C223" s="3"/>
+      <c r="D223" s="4"/>
       <c r="E223" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -6301,6 +6542,7 @@
         <v/>
       </c>
       <c r="C224" s="3"/>
+      <c r="D224" s="4"/>
       <c r="E224" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -6324,6 +6566,7 @@
         <v/>
       </c>
       <c r="C225" s="3"/>
+      <c r="D225" s="4"/>
       <c r="E225" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -6347,6 +6590,7 @@
         <v/>
       </c>
       <c r="C226" s="3"/>
+      <c r="D226" s="4"/>
       <c r="E226" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -6370,6 +6614,7 @@
         <v/>
       </c>
       <c r="C227" s="3"/>
+      <c r="D227" s="4"/>
       <c r="E227" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -6393,6 +6638,7 @@
         <v/>
       </c>
       <c r="C228" s="3"/>
+      <c r="D228" s="4"/>
       <c r="E228" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -6416,6 +6662,7 @@
         <v/>
       </c>
       <c r="C229" s="3"/>
+      <c r="D229" s="4"/>
       <c r="E229" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -6439,6 +6686,7 @@
         <v/>
       </c>
       <c r="C230" s="3"/>
+      <c r="D230" s="4"/>
       <c r="E230" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -6462,6 +6710,7 @@
         <v/>
       </c>
       <c r="C231" s="3"/>
+      <c r="D231" s="4"/>
       <c r="E231" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -6485,6 +6734,7 @@
         <v/>
       </c>
       <c r="C232" s="3"/>
+      <c r="D232" s="4"/>
       <c r="E232" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -6508,6 +6758,7 @@
         <v/>
       </c>
       <c r="C233" s="3"/>
+      <c r="D233" s="4"/>
       <c r="E233" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -6531,6 +6782,7 @@
         <v/>
       </c>
       <c r="C234" s="3"/>
+      <c r="D234" s="4"/>
       <c r="E234" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -6554,6 +6806,7 @@
         <v/>
       </c>
       <c r="C235" s="3"/>
+      <c r="D235" s="4"/>
       <c r="E235" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -6577,6 +6830,7 @@
         <v/>
       </c>
       <c r="C236" s="3"/>
+      <c r="D236" s="4"/>
       <c r="E236" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -6600,6 +6854,7 @@
         <v/>
       </c>
       <c r="C237" s="3"/>
+      <c r="D237" s="4"/>
       <c r="E237" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -6623,6 +6878,7 @@
         <v/>
       </c>
       <c r="C238" s="3"/>
+      <c r="D238" s="4"/>
       <c r="E238" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -6646,6 +6902,7 @@
         <v/>
       </c>
       <c r="C239" s="3"/>
+      <c r="D239" s="4"/>
       <c r="E239" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -6669,6 +6926,7 @@
         <v/>
       </c>
       <c r="C240" s="3"/>
+      <c r="D240" s="4"/>
       <c r="E240" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -6692,6 +6950,7 @@
         <v/>
       </c>
       <c r="C241" s="3"/>
+      <c r="D241" s="4"/>
       <c r="E241" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -6715,6 +6974,7 @@
         <v/>
       </c>
       <c r="C242" s="3"/>
+      <c r="D242" s="4"/>
       <c r="E242" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -6738,6 +6998,7 @@
         <v/>
       </c>
       <c r="C243" s="3"/>
+      <c r="D243" s="4"/>
       <c r="E243" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -6761,6 +7022,7 @@
         <v/>
       </c>
       <c r="C244" s="3"/>
+      <c r="D244" s="4"/>
       <c r="E244" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -6784,6 +7046,7 @@
         <v/>
       </c>
       <c r="C245" s="3"/>
+      <c r="D245" s="4"/>
       <c r="E245" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -6807,6 +7070,7 @@
         <v/>
       </c>
       <c r="C246" s="3"/>
+      <c r="D246" s="4"/>
       <c r="E246" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -6830,6 +7094,7 @@
         <v/>
       </c>
       <c r="C247" s="3"/>
+      <c r="D247" s="4"/>
       <c r="E247" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -6853,6 +7118,7 @@
         <v/>
       </c>
       <c r="C248" s="3"/>
+      <c r="D248" s="4"/>
       <c r="E248" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -6876,6 +7142,7 @@
         <v/>
       </c>
       <c r="C249" s="3"/>
+      <c r="D249" s="4"/>
       <c r="E249" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -6899,6 +7166,7 @@
         <v/>
       </c>
       <c r="C250" s="3"/>
+      <c r="D250" s="4"/>
       <c r="E250" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -6922,6 +7190,7 @@
         <v/>
       </c>
       <c r="C251" s="3"/>
+      <c r="D251" s="4"/>
       <c r="E251" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -6945,6 +7214,7 @@
         <v/>
       </c>
       <c r="C252" s="3"/>
+      <c r="D252" s="4"/>
       <c r="E252" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -6968,6 +7238,7 @@
         <v/>
       </c>
       <c r="C253" s="3"/>
+      <c r="D253" s="4"/>
       <c r="E253" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -6991,6 +7262,7 @@
         <v/>
       </c>
       <c r="C254" s="3"/>
+      <c r="D254" s="4"/>
       <c r="E254" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -7014,6 +7286,7 @@
         <v/>
       </c>
       <c r="C255" s="3"/>
+      <c r="D255" s="4"/>
       <c r="E255" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -7037,6 +7310,7 @@
         <v/>
       </c>
       <c r="C256" s="3"/>
+      <c r="D256" s="4"/>
       <c r="E256" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -7060,6 +7334,7 @@
         <v/>
       </c>
       <c r="C257" s="3"/>
+      <c r="D257" s="4"/>
       <c r="E257" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -7083,6 +7358,7 @@
         <v/>
       </c>
       <c r="C258" s="3"/>
+      <c r="D258" s="4"/>
       <c r="E258" t="str">
         <f t="shared" si="3"/>
         <v/>
@@ -7106,6 +7382,7 @@
         <v/>
       </c>
       <c r="C259" s="3"/>
+      <c r="D259" s="4"/>
       <c r="E259" t="str">
         <f t="shared" ref="E259:E322" si="4">IF(F259="","",IF(F259="water_draw","water_draw",IF(F259="end","test","cta")))</f>
         <v/>
@@ -7129,6 +7406,7 @@
         <v/>
       </c>
       <c r="C260" s="3"/>
+      <c r="D260" s="4"/>
       <c r="E260" t="str">
         <f t="shared" si="4"/>
         <v/>
@@ -7152,6 +7430,7 @@
         <v/>
       </c>
       <c r="C261" s="3"/>
+      <c r="D261" s="4"/>
       <c r="E261" t="str">
         <f t="shared" si="4"/>
         <v/>
@@ -7175,6 +7454,7 @@
         <v/>
       </c>
       <c r="C262" s="3"/>
+      <c r="D262" s="4"/>
       <c r="E262" t="str">
         <f t="shared" si="4"/>
         <v/>
@@ -7198,6 +7478,7 @@
         <v/>
       </c>
       <c r="C263" s="3"/>
+      <c r="D263" s="4"/>
       <c r="E263" t="str">
         <f t="shared" si="4"/>
         <v/>
@@ -7221,6 +7502,7 @@
         <v/>
       </c>
       <c r="C264" s="3"/>
+      <c r="D264" s="4"/>
       <c r="E264" t="str">
         <f t="shared" si="4"/>
         <v/>
@@ -7244,6 +7526,7 @@
         <v/>
       </c>
       <c r="C265" s="3"/>
+      <c r="D265" s="4"/>
       <c r="E265" t="str">
         <f t="shared" si="4"/>
         <v/>
@@ -7267,6 +7550,7 @@
         <v/>
       </c>
       <c r="C266" s="3"/>
+      <c r="D266" s="4"/>
       <c r="E266" t="str">
         <f t="shared" si="4"/>
         <v/>
@@ -7290,6 +7574,7 @@
         <v/>
       </c>
       <c r="C267" s="3"/>
+      <c r="D267" s="4"/>
       <c r="E267" t="str">
         <f t="shared" si="4"/>
         <v/>
@@ -7313,6 +7598,7 @@
         <v/>
       </c>
       <c r="C268" s="3"/>
+      <c r="D268" s="4"/>
       <c r="E268" t="str">
         <f t="shared" si="4"/>
         <v/>
@@ -7336,6 +7622,7 @@
         <v/>
       </c>
       <c r="C269" s="3"/>
+      <c r="D269" s="4"/>
       <c r="E269" t="str">
         <f t="shared" si="4"/>
         <v/>
@@ -7359,6 +7646,7 @@
         <v/>
       </c>
       <c r="C270" s="3"/>
+      <c r="D270" s="4"/>
       <c r="E270" t="str">
         <f t="shared" si="4"/>
         <v/>
@@ -7382,6 +7670,7 @@
         <v/>
       </c>
       <c r="C271" s="3"/>
+      <c r="D271" s="4"/>
       <c r="E271" t="str">
         <f t="shared" si="4"/>
         <v/>
@@ -7405,6 +7694,7 @@
         <v/>
       </c>
       <c r="C272" s="3"/>
+      <c r="D272" s="4"/>
       <c r="E272" t="str">
         <f t="shared" si="4"/>
         <v/>
@@ -7428,6 +7718,7 @@
         <v/>
       </c>
       <c r="C273" s="3"/>
+      <c r="D273" s="4"/>
       <c r="E273" t="str">
         <f t="shared" si="4"/>
         <v/>
@@ -7451,6 +7742,7 @@
         <v/>
       </c>
       <c r="C274" s="3"/>
+      <c r="D274" s="4"/>
       <c r="E274" t="str">
         <f t="shared" si="4"/>
         <v/>
@@ -7474,6 +7766,7 @@
         <v/>
       </c>
       <c r="C275" s="3"/>
+      <c r="D275" s="4"/>
       <c r="E275" t="str">
         <f t="shared" si="4"/>
         <v/>
@@ -7497,6 +7790,7 @@
         <v/>
       </c>
       <c r="C276" s="3"/>
+      <c r="D276" s="4"/>
       <c r="E276" t="str">
         <f t="shared" si="4"/>
         <v/>
@@ -7520,6 +7814,7 @@
         <v/>
       </c>
       <c r="C277" s="3"/>
+      <c r="D277" s="4"/>
       <c r="E277" t="str">
         <f t="shared" si="4"/>
         <v/>
@@ -7543,6 +7838,7 @@
         <v/>
       </c>
       <c r="C278" s="3"/>
+      <c r="D278" s="4"/>
       <c r="E278" t="str">
         <f t="shared" si="4"/>
         <v/>
@@ -7566,6 +7862,7 @@
         <v/>
       </c>
       <c r="C279" s="3"/>
+      <c r="D279" s="4"/>
       <c r="E279" t="str">
         <f t="shared" si="4"/>
         <v/>
@@ -7589,6 +7886,7 @@
         <v/>
       </c>
       <c r="C280" s="3"/>
+      <c r="D280" s="4"/>
       <c r="E280" t="str">
         <f t="shared" si="4"/>
         <v/>
@@ -7612,6 +7910,7 @@
         <v/>
       </c>
       <c r="C281" s="3"/>
+      <c r="D281" s="4"/>
       <c r="E281" t="str">
         <f t="shared" si="4"/>
         <v/>
@@ -7635,6 +7934,7 @@
         <v/>
       </c>
       <c r="C282" s="3"/>
+      <c r="D282" s="4"/>
       <c r="E282" t="str">
         <f t="shared" si="4"/>
         <v/>
@@ -7658,6 +7958,7 @@
         <v/>
       </c>
       <c r="C283" s="3"/>
+      <c r="D283" s="4"/>
       <c r="E283" t="str">
         <f t="shared" si="4"/>
         <v/>
@@ -7681,6 +7982,7 @@
         <v/>
       </c>
       <c r="C284" s="3"/>
+      <c r="D284" s="4"/>
       <c r="E284" t="str">
         <f t="shared" si="4"/>
         <v/>
@@ -7704,6 +8006,7 @@
         <v/>
       </c>
       <c r="C285" s="3"/>
+      <c r="D285" s="4"/>
       <c r="E285" t="str">
         <f t="shared" si="4"/>
         <v/>
@@ -7727,6 +8030,7 @@
         <v/>
       </c>
       <c r="C286" s="3"/>
+      <c r="D286" s="4"/>
       <c r="E286" t="str">
         <f t="shared" si="4"/>
         <v/>
@@ -7750,6 +8054,7 @@
         <v/>
       </c>
       <c r="C287" s="3"/>
+      <c r="D287" s="4"/>
       <c r="E287" t="str">
         <f t="shared" si="4"/>
         <v/>
@@ -7773,6 +8078,7 @@
         <v/>
       </c>
       <c r="C288" s="3"/>
+      <c r="D288" s="4"/>
       <c r="E288" t="str">
         <f t="shared" si="4"/>
         <v/>
@@ -7796,6 +8102,7 @@
         <v/>
       </c>
       <c r="C289" s="3"/>
+      <c r="D289" s="4"/>
       <c r="E289" t="str">
         <f t="shared" si="4"/>
         <v/>
@@ -7819,6 +8126,7 @@
         <v/>
       </c>
       <c r="C290" s="3"/>
+      <c r="D290" s="4"/>
       <c r="E290" t="str">
         <f t="shared" si="4"/>
         <v/>
@@ -7842,6 +8150,7 @@
         <v/>
       </c>
       <c r="C291" s="3"/>
+      <c r="D291" s="4"/>
       <c r="E291" t="str">
         <f t="shared" si="4"/>
         <v/>
@@ -7865,6 +8174,7 @@
         <v/>
       </c>
       <c r="C292" s="3"/>
+      <c r="D292" s="4"/>
       <c r="E292" t="str">
         <f t="shared" si="4"/>
         <v/>
@@ -7888,6 +8198,7 @@
         <v/>
       </c>
       <c r="C293" s="3"/>
+      <c r="D293" s="4"/>
       <c r="E293" t="str">
         <f t="shared" si="4"/>
         <v/>
@@ -7911,6 +8222,7 @@
         <v/>
       </c>
       <c r="C294" s="3"/>
+      <c r="D294" s="4"/>
       <c r="E294" t="str">
         <f t="shared" si="4"/>
         <v/>
@@ -7934,6 +8246,7 @@
         <v/>
       </c>
       <c r="C295" s="3"/>
+      <c r="D295" s="4"/>
       <c r="E295" t="str">
         <f t="shared" si="4"/>
         <v/>
@@ -7957,6 +8270,7 @@
         <v/>
       </c>
       <c r="C296" s="3"/>
+      <c r="D296" s="4"/>
       <c r="E296" t="str">
         <f t="shared" si="4"/>
         <v/>
@@ -7980,6 +8294,7 @@
         <v/>
       </c>
       <c r="C297" s="3"/>
+      <c r="D297" s="4"/>
       <c r="E297" t="str">
         <f t="shared" si="4"/>
         <v/>
@@ -8003,6 +8318,7 @@
         <v/>
       </c>
       <c r="C298" s="3"/>
+      <c r="D298" s="4"/>
       <c r="E298" t="str">
         <f t="shared" si="4"/>
         <v/>
@@ -8026,6 +8342,7 @@
         <v/>
       </c>
       <c r="C299" s="3"/>
+      <c r="D299" s="4"/>
       <c r="E299" t="str">
         <f t="shared" si="4"/>
         <v/>
@@ -8049,6 +8366,7 @@
         <v/>
       </c>
       <c r="C300" s="3"/>
+      <c r="D300" s="4"/>
       <c r="E300" t="str">
         <f t="shared" si="4"/>
         <v/>
@@ -8072,6 +8390,7 @@
         <v/>
       </c>
       <c r="C301" s="3"/>
+      <c r="D301" s="4"/>
       <c r="E301" t="str">
         <f t="shared" si="4"/>
         <v/>
@@ -8095,6 +8414,7 @@
         <v/>
       </c>
       <c r="C302" s="3"/>
+      <c r="D302" s="4"/>
       <c r="E302" t="str">
         <f t="shared" si="4"/>
         <v/>
@@ -8118,6 +8438,7 @@
         <v/>
       </c>
       <c r="C303" s="3"/>
+      <c r="D303" s="4"/>
       <c r="E303" t="str">
         <f t="shared" si="4"/>
         <v/>
@@ -8141,6 +8462,7 @@
         <v/>
       </c>
       <c r="C304" s="3"/>
+      <c r="D304" s="4"/>
       <c r="E304" t="str">
         <f t="shared" si="4"/>
         <v/>
@@ -8164,6 +8486,7 @@
         <v/>
       </c>
       <c r="C305" s="3"/>
+      <c r="D305" s="4"/>
       <c r="E305" t="str">
         <f t="shared" si="4"/>
         <v/>
@@ -8187,6 +8510,7 @@
         <v/>
       </c>
       <c r="C306" s="3"/>
+      <c r="D306" s="4"/>
       <c r="E306" t="str">
         <f t="shared" si="4"/>
         <v/>
@@ -8210,6 +8534,7 @@
         <v/>
       </c>
       <c r="C307" s="3"/>
+      <c r="D307" s="4"/>
       <c r="E307" t="str">
         <f t="shared" si="4"/>
         <v/>
@@ -8233,6 +8558,7 @@
         <v/>
       </c>
       <c r="C308" s="3"/>
+      <c r="D308" s="4"/>
       <c r="E308" t="str">
         <f t="shared" si="4"/>
         <v/>
@@ -8256,6 +8582,7 @@
         <v/>
       </c>
       <c r="C309" s="3"/>
+      <c r="D309" s="4"/>
       <c r="E309" t="str">
         <f t="shared" si="4"/>
         <v/>
@@ -8279,6 +8606,7 @@
         <v/>
       </c>
       <c r="C310" s="3"/>
+      <c r="D310" s="4"/>
       <c r="E310" t="str">
         <f t="shared" si="4"/>
         <v/>
@@ -8302,6 +8630,7 @@
         <v/>
       </c>
       <c r="C311" s="3"/>
+      <c r="D311" s="4"/>
       <c r="E311" t="str">
         <f t="shared" si="4"/>
         <v/>
@@ -8325,6 +8654,7 @@
         <v/>
       </c>
       <c r="C312" s="3"/>
+      <c r="D312" s="4"/>
       <c r="E312" t="str">
         <f t="shared" si="4"/>
         <v/>
@@ -8348,6 +8678,7 @@
         <v/>
       </c>
       <c r="C313" s="3"/>
+      <c r="D313" s="4"/>
       <c r="E313" t="str">
         <f t="shared" si="4"/>
         <v/>
@@ -8371,6 +8702,7 @@
         <v/>
       </c>
       <c r="C314" s="3"/>
+      <c r="D314" s="4"/>
       <c r="E314" t="str">
         <f t="shared" si="4"/>
         <v/>
@@ -8394,6 +8726,7 @@
         <v/>
       </c>
       <c r="C315" s="3"/>
+      <c r="D315" s="4"/>
       <c r="E315" t="str">
         <f t="shared" si="4"/>
         <v/>
@@ -8417,6 +8750,7 @@
         <v/>
       </c>
       <c r="C316" s="3"/>
+      <c r="D316" s="4"/>
       <c r="E316" t="str">
         <f t="shared" si="4"/>
         <v/>
@@ -8440,6 +8774,7 @@
         <v/>
       </c>
       <c r="C317" s="3"/>
+      <c r="D317" s="4"/>
       <c r="E317" t="str">
         <f t="shared" si="4"/>
         <v/>
@@ -8463,6 +8798,7 @@
         <v/>
       </c>
       <c r="C318" s="3"/>
+      <c r="D318" s="4"/>
       <c r="E318" t="str">
         <f t="shared" si="4"/>
         <v/>
@@ -8486,6 +8822,7 @@
         <v/>
       </c>
       <c r="C319" s="3"/>
+      <c r="D319" s="4"/>
       <c r="E319" t="str">
         <f t="shared" si="4"/>
         <v/>
@@ -8509,6 +8846,7 @@
         <v/>
       </c>
       <c r="C320" s="3"/>
+      <c r="D320" s="4"/>
       <c r="E320" t="str">
         <f t="shared" si="4"/>
         <v/>
@@ -8532,6 +8870,7 @@
         <v/>
       </c>
       <c r="C321" s="3"/>
+      <c r="D321" s="4"/>
       <c r="E321" t="str">
         <f t="shared" si="4"/>
         <v/>
@@ -8555,6 +8894,7 @@
         <v/>
       </c>
       <c r="C322" s="3"/>
+      <c r="D322" s="4"/>
       <c r="E322" t="str">
         <f t="shared" si="4"/>
         <v/>
@@ -8578,6 +8918,7 @@
         <v/>
       </c>
       <c r="C323" s="3"/>
+      <c r="D323" s="4"/>
       <c r="E323" t="str">
         <f t="shared" ref="E323:E336" si="5">IF(F323="","",IF(F323="water_draw","water_draw",IF(F323="end","test","cta")))</f>
         <v/>
@@ -8601,6 +8942,7 @@
         <v/>
       </c>
       <c r="C324" s="3"/>
+      <c r="D324" s="4"/>
       <c r="E324" t="str">
         <f t="shared" si="5"/>
         <v/>
@@ -8624,6 +8966,7 @@
         <v/>
       </c>
       <c r="C325" s="3"/>
+      <c r="D325" s="4"/>
       <c r="E325" t="str">
         <f t="shared" si="5"/>
         <v/>
@@ -8647,6 +8990,7 @@
         <v/>
       </c>
       <c r="C326" s="3"/>
+      <c r="D326" s="4"/>
       <c r="E326" t="str">
         <f t="shared" si="5"/>
         <v/>
@@ -8670,6 +9014,7 @@
         <v/>
       </c>
       <c r="C327" s="3"/>
+      <c r="D327" s="4"/>
       <c r="E327" t="str">
         <f t="shared" si="5"/>
         <v/>
@@ -8693,6 +9038,7 @@
         <v/>
       </c>
       <c r="C328" s="3"/>
+      <c r="D328" s="4"/>
       <c r="E328" t="str">
         <f t="shared" si="5"/>
         <v/>
@@ -8716,6 +9062,7 @@
         <v/>
       </c>
       <c r="C329" s="3"/>
+      <c r="D329" s="4"/>
       <c r="E329" t="str">
         <f t="shared" si="5"/>
         <v/>
@@ -8739,6 +9086,7 @@
         <v/>
       </c>
       <c r="C330" s="3"/>
+      <c r="D330" s="4"/>
       <c r="E330" t="str">
         <f t="shared" si="5"/>
         <v/>
@@ -8762,6 +9110,7 @@
         <v/>
       </c>
       <c r="C331" s="3"/>
+      <c r="D331" s="4"/>
       <c r="E331" t="str">
         <f t="shared" si="5"/>
         <v/>
@@ -8785,6 +9134,7 @@
         <v/>
       </c>
       <c r="C332" s="3"/>
+      <c r="D332" s="4"/>
       <c r="E332" t="str">
         <f t="shared" si="5"/>
         <v/>
@@ -8808,6 +9158,7 @@
         <v/>
       </c>
       <c r="C333" s="3"/>
+      <c r="D333" s="4"/>
       <c r="E333" t="str">
         <f t="shared" si="5"/>
         <v/>
@@ -8831,6 +9182,7 @@
         <v/>
       </c>
       <c r="C334" s="3"/>
+      <c r="D334" s="4"/>
       <c r="E334" t="str">
         <f t="shared" si="5"/>
         <v/>
@@ -8854,6 +9206,7 @@
         <v/>
       </c>
       <c r="C335" s="3"/>
+      <c r="D335" s="4"/>
       <c r="E335" t="str">
         <f t="shared" si="5"/>
         <v/>
@@ -8877,6 +9230,7 @@
         <v/>
       </c>
       <c r="C336" s="4"/>
+      <c r="D336" s="4"/>
       <c r="E336" t="str">
         <f t="shared" si="5"/>
         <v/>
@@ -8895,7 +9249,7 @@
     </row>
   </sheetData>
   <sheetProtection sheet="1" objects="1" scenarios="1"/>
-  <dataValidations xWindow="374" yWindow="509" count="10">
+  <dataValidations xWindow="853" yWindow="532" count="9">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid schedule value" error="Enter a value allowed for this schedule field." promptTitle="Action" prompt="The CTA-2045 command you want the run from the dropdown menu" sqref="F2:F336" xr:uid="{8634ECE3-E7CB-4581-95B1-4AB9629A7C09}">
       <formula1>"advanced_load_up,critical_peak,end,grid_emergency,load_up,run_normal,shed,water_draw"</formula1>
     </dataValidation>
@@ -8922,10 +9276,7 @@
     <dataValidation type="decimal" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid schedule value" error="Enter a value allowed for this schedule field." promptTitle="Water volume" prompt="For a water draw, enter the target volume in gallons as a positive number." sqref="K2:K336" xr:uid="{20C96F37-19E2-47CC-8AA8-74594A30CE50}">
       <formula1>0</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Phase" prompt="Which phase of the event is this?" sqref="D2:D9" xr:uid="{B7A1C4F3-E440-47ED-8265-ED7C15FCA655}">
-      <formula1>"event,pre_event,recovery"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Phase" prompt="Which phase of the event is this?" sqref="D10:D336" xr:uid="{FD1C2215-35ED-410F-ABB3-AAA8065ABA9C}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Phase" prompt="Which phase of the event is this?" sqref="D2:D336" xr:uid="{B7A1C4F3-E440-47ED-8265-ED7C15FCA655}">
       <formula1>"event,pre_event,recovery"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
updated mandatory fields that were blank in the scheduler
</commit_message>
<xml_diff>
--- a/software/conformance_test_schedule_main.xlsx
+++ b/software/conformance_test_schedule_main.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pwrgra09-admin\Documents\myPythonFiles\Root\conformance_testing_team\software\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D33C12C4-333F-4CD7-8590-3132D55C2F65}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A0CEE6D3-EB39-4077-B0BD-D928CC11788D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="15720" xr2:uid="{C8C0DF4B-6D5B-4BD3-847D-4558E3821A3D}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="36">
   <si>
     <t>enabled</t>
   </si>
@@ -140,6 +140,9 @@
   </si>
   <si>
     <t>Attemp Advanced Load up</t>
+  </si>
+  <si>
+    <t>100_wh</t>
   </si>
 </sst>
 </file>
@@ -1389,8 +1392,12 @@
       <c r="G10" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="H10" s="4"/>
-      <c r="I10" s="4"/>
+      <c r="H10" s="4">
+        <v>5</v>
+      </c>
+      <c r="I10" s="4" t="s">
+        <v>35</v>
+      </c>
       <c r="J10" s="2" t="str">
         <f>IFERROR(_xlfn.XLOOKUP(F10,'CTA Actions'!$A$2:$A$7,'CTA Actions'!$B$2:$B$7),"")</f>
         <v>3|6</v>

</xml_diff>

<commit_message>
updated a new schedule to test
</commit_message>
<xml_diff>
--- a/software/conformance_test_schedule_main.xlsx
+++ b/software/conformance_test_schedule_main.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pwrgra09-admin\Documents\myPythonFiles\Root\conformance_testing_team\software\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A0CEE6D3-EB39-4077-B0BD-D928CC11788D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BFE449EF-22A3-46AC-9C20-7C906F74BE7D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="15720" xr2:uid="{C8C0DF4B-6D5B-4BD3-847D-4558E3821A3D}"/>
+    <workbookView xWindow="38280" yWindow="-120" windowWidth="25440" windowHeight="15270" xr2:uid="{C8C0DF4B-6D5B-4BD3-847D-4558E3821A3D}"/>
   </bookViews>
   <sheets>
     <sheet name="conformance_test_schedule_main" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="36">
   <si>
     <t>enabled</t>
   </si>
@@ -1086,7 +1086,7 @@
       </c>
       <c r="B2" t="str">
         <f>IF(F2="","",IF(F2="end","test_end",F2&amp;"_"&amp;COUNTIF($F$2:F2,F2)))</f>
-        <v>load_up_1</v>
+        <v>shed_1</v>
       </c>
       <c r="C2" s="3">
         <v>0</v>
@@ -1099,16 +1099,16 @@
         <v>cta</v>
       </c>
       <c r="F2" s="4" t="s">
-        <v>13</v>
+        <v>28</v>
       </c>
       <c r="G2" s="4">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H2" s="4"/>
       <c r="I2" s="4"/>
       <c r="J2" s="2" t="str">
         <f>IFERROR(_xlfn.XLOOKUP(F2,'CTA Actions'!$A$2:$A$7,'CTA Actions'!$B$2:$B$7),"")</f>
-        <v>3|6</v>
+        <v>2|4</v>
       </c>
       <c r="K2" s="4"/>
       <c r="L2" s="4"/>
@@ -1122,10 +1122,10 @@
       </c>
       <c r="B3" t="str">
         <f>IF(F3="","",IF(F3="end","test_end",F3&amp;"_"&amp;COUNTIF($F$2:F3,F3)))</f>
-        <v>run_normal_1</v>
+        <v>advanced_load_up_1</v>
       </c>
       <c r="C3" s="3">
-        <v>4.8611111111111112E-3</v>
+        <v>2.0833333333333333E-3</v>
       </c>
       <c r="D3" s="4" t="s">
         <v>20</v>
@@ -1135,16 +1135,20 @@
         <v>cta</v>
       </c>
       <c r="F3" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="G3" s="4">
-        <v>3</v>
-      </c>
-      <c r="H3" s="4"/>
-      <c r="I3" s="4"/>
+        <v>25</v>
+      </c>
+      <c r="G3" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="H3" s="4">
+        <v>5</v>
+      </c>
+      <c r="I3" s="4" t="s">
+        <v>35</v>
+      </c>
       <c r="J3" s="2" t="str">
         <f>IFERROR(_xlfn.XLOOKUP(F3,'CTA Actions'!$A$2:$A$7,'CTA Actions'!$B$2:$B$7),"")</f>
-        <v>1|0</v>
+        <v>3|6</v>
       </c>
       <c r="K3" s="4"/>
       <c r="L3" s="4"/>
@@ -1158,10 +1162,10 @@
       </c>
       <c r="B4" t="str">
         <f>IF(F4="","",IF(F4="end","test_end",F4&amp;"_"&amp;COUNTIF($F$2:F4,F4)))</f>
-        <v>critical_peak_1</v>
+        <v>run_normal_1</v>
       </c>
       <c r="C4" s="3">
-        <v>8.3333333333333332E-3</v>
+        <v>4.1666666666666666E-3</v>
       </c>
       <c r="D4" s="4" t="s">
         <v>16</v>
@@ -1171,7 +1175,7 @@
         <v>cta</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>26</v>
+        <v>17</v>
       </c>
       <c r="G4" s="4">
         <v>7</v>
@@ -1180,7 +1184,7 @@
       <c r="I4" s="4"/>
       <c r="J4" s="2" t="str">
         <f>IFERROR(_xlfn.XLOOKUP(F4,'CTA Actions'!$A$2:$A$7,'CTA Actions'!$B$2:$B$7),"")</f>
-        <v>2|4</v>
+        <v>1|0</v>
       </c>
       <c r="K4" s="4"/>
       <c r="L4" s="4"/>
@@ -1194,7 +1198,7 @@
       </c>
       <c r="B5" t="str">
         <f>IF(F5="","",IF(F5="end","test_end",F5&amp;"_"&amp;COUNTIF($F$2:F5,F5)))</f>
-        <v>run_normal_2</v>
+        <v>test_end</v>
       </c>
       <c r="C5" s="3">
         <v>1.5277777777777777E-2</v>
@@ -1204,10 +1208,10 @@
       </c>
       <c r="E5" t="str">
         <f t="shared" si="0"/>
-        <v>cta</v>
+        <v>test</v>
       </c>
       <c r="F5" s="4" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="G5" s="4" t="s">
         <v>18</v>
@@ -1216,7 +1220,7 @@
       <c r="I5" s="4"/>
       <c r="J5" s="2" t="str">
         <f>IFERROR(_xlfn.XLOOKUP(F5,'CTA Actions'!$A$2:$A$7,'CTA Actions'!$B$2:$B$7),"")</f>
-        <v>1|0</v>
+        <v/>
       </c>
       <c r="K5" s="4"/>
       <c r="L5" s="4"/>
@@ -1226,11 +1230,11 @@
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B6" t="str">
         <f>IF(F6="","",IF(F6="end","test_end",F6&amp;"_"&amp;COUNTIF($F$2:F6,F6)))</f>
-        <v>shed_1</v>
+        <v>shed_2</v>
       </c>
       <c r="C6" s="3">
         <v>1.7361111111111112E-2</v>
@@ -1262,11 +1266,11 @@
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B7" t="str">
         <f>IF(F7="","",IF(F7="end","test_end",F7&amp;"_"&amp;COUNTIF($F$2:F7,F7)))</f>
-        <v>run_normal_3</v>
+        <v>run_normal_2</v>
       </c>
       <c r="C7" s="3">
         <v>2.4305555555555556E-2</v>
@@ -1298,7 +1302,7 @@
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A8" s="4" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B8" t="str">
         <f>IF(F8="","",IF(F8="end","test_end",F8&amp;"_"&amp;COUNTIF($F$2:F8,F8)))</f>
@@ -1334,11 +1338,11 @@
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A9" s="4" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B9" t="str">
         <f>IF(F9="","",IF(F9="end","test_end",F9&amp;"_"&amp;COUNTIF($F$2:F9,F9)))</f>
-        <v>run_normal_4</v>
+        <v>run_normal_3</v>
       </c>
       <c r="C9" s="3">
         <v>3.2638888888888891E-2</v>
@@ -1370,11 +1374,11 @@
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A10" s="4" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B10" t="str">
         <f>IF(F10="","",IF(F10="end","test_end",F10&amp;"_"&amp;COUNTIF($F$2:F10,F10)))</f>
-        <v>advanced_load_up_1</v>
+        <v>advanced_load_up_2</v>
       </c>
       <c r="C10" s="3">
         <v>3.4027777777777775E-2</v>
@@ -1410,11 +1414,11 @@
     </row>
     <row r="11" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A11" s="4" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B11" t="str">
         <f>IF(F11="","",IF(F11="end","test_end",F11&amp;"_"&amp;COUNTIF($F$2:F11,F11)))</f>
-        <v>run_normal_5</v>
+        <v>run_normal_4</v>
       </c>
       <c r="C11" s="3">
         <v>3.5416666666666666E-2</v>
@@ -1453,7 +1457,7 @@
         <v>test_end</v>
       </c>
       <c r="C12" s="3">
-        <v>3.6805555555555557E-2</v>
+        <v>5.5555555555555558E-3</v>
       </c>
       <c r="D12" s="4" t="s">
         <v>20</v>
@@ -9256,7 +9260,7 @@
     </row>
   </sheetData>
   <sheetProtection sheet="1" objects="1" scenarios="1"/>
-  <dataValidations xWindow="853" yWindow="532" count="9">
+  <dataValidations xWindow="256" yWindow="493" count="9">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid schedule value" error="Enter a value allowed for this schedule field." promptTitle="Action" prompt="The CTA-2045 command you want the run from the dropdown menu" sqref="F2:F336" xr:uid="{8634ECE3-E7CB-4581-95B1-4AB9629A7C09}">
       <formula1>"advanced_load_up,critical_peak,end,grid_emergency,load_up,run_normal,shed,water_draw"</formula1>
     </dataValidation>

</xml_diff>

<commit_message>
update the scheduler to manage water sensor calibration
</commit_message>
<xml_diff>
--- a/software/conformance_test_schedule_main.xlsx
+++ b/software/conformance_test_schedule_main.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pwrgra09-admin\Documents\myPythonFiles\Root\conformance_testing_team\software\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6FBDB812-359B-439E-B9E5-1FA64BE441C1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F58DDA62-622C-45E5-8AD5-73BABD2C484F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38190" yWindow="4185" windowWidth="25410" windowHeight="11295" xr2:uid="{C8C0DF4B-6D5B-4BD3-847D-4558E3821A3D}"/>
+    <workbookView xWindow="38190" yWindow="1170" windowWidth="25410" windowHeight="11295" xr2:uid="{C8C0DF4B-6D5B-4BD3-847D-4558E3821A3D}"/>
   </bookViews>
   <sheets>
     <sheet name="conformance_test_schedule_main" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="38">
   <si>
     <t>enabled</t>
   </si>
@@ -146,6 +146,9 @@
   </si>
   <si>
     <t>return to normal</t>
+  </si>
+  <si>
+    <t>water_draw</t>
   </si>
 </sst>
 </file>
@@ -1104,8 +1107,8 @@
       <c r="F2" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="G2" s="4">
-        <v>3</v>
+      <c r="G2" s="4" t="s">
+        <v>17</v>
       </c>
       <c r="H2" s="4"/>
       <c r="I2" s="4"/>
@@ -1180,8 +1183,8 @@
       <c r="F4" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="G4" s="4">
-        <v>7</v>
+      <c r="G4" s="4" t="s">
+        <v>17</v>
       </c>
       <c r="H4" s="4"/>
       <c r="I4" s="4"/>
@@ -1197,14 +1200,14 @@
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B5" t="str">
         <f>IF(F5="","",IF(F5="end","test_end",F5&amp;"_"&amp;COUNTIF($F$2:F5,F5)))</f>
         <v>load_up_1</v>
       </c>
       <c r="C5" s="3">
-        <v>1.5277777777777777E-2</v>
+        <v>5.5555555555555558E-3</v>
       </c>
       <c r="D5" s="4" t="s">
         <v>19</v>
@@ -1233,14 +1236,14 @@
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B6" t="str">
         <f>IF(F6="","",IF(F6="end","test_end",F6&amp;"_"&amp;COUNTIF($F$2:F6,F6)))</f>
         <v>shed_2</v>
       </c>
       <c r="C6" s="3">
-        <v>1.7361111111111112E-2</v>
+        <v>9.7222222222222224E-3</v>
       </c>
       <c r="D6" s="4" t="s">
         <v>15</v>
@@ -1252,8 +1255,8 @@
       <c r="F6" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="G6" s="4">
-        <v>5</v>
+      <c r="G6" s="4" t="s">
+        <v>17</v>
       </c>
       <c r="H6" s="4"/>
       <c r="I6" s="4"/>
@@ -1269,50 +1272,52 @@
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B7" t="str">
         <f>IF(F7="","",IF(F7="end","test_end",F7&amp;"_"&amp;COUNTIF($F$2:F7,F7)))</f>
-        <v>run_normal_2</v>
+        <v>water_draw_1</v>
       </c>
       <c r="C7" s="3">
-        <v>2.4305555555555556E-2</v>
+        <v>1.1111111111111112E-2</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="E7" t="str">
         <f t="shared" si="0"/>
-        <v>cta</v>
+        <v>water_draw</v>
       </c>
       <c r="F7" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="G7" s="4" t="s">
-        <v>17</v>
-      </c>
+        <v>37</v>
+      </c>
+      <c r="G7" s="4"/>
       <c r="H7" s="4"/>
       <c r="I7" s="4"/>
       <c r="J7" s="2" t="str">
         <f>IFERROR(_xlfn.XLOOKUP(F7,'CTA Actions'!$A$2:$A$7,'CTA Actions'!$B$2:$B$7),"")</f>
-        <v>1|0</v>
-      </c>
-      <c r="K7" s="4"/>
-      <c r="L7" s="4"/>
+        <v/>
+      </c>
+      <c r="K7" s="4">
+        <v>9</v>
+      </c>
+      <c r="L7" s="4">
+        <v>3</v>
+      </c>
       <c r="M7" s="4" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A8" s="4" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B8" t="str">
         <f>IF(F8="","",IF(F8="end","test_end",F8&amp;"_"&amp;COUNTIF($F$2:F8,F8)))</f>
         <v>grid_emergency_1</v>
       </c>
       <c r="C8" s="3">
-        <v>2.5694444444444443E-2</v>
+        <v>1.4583333333333334E-2</v>
       </c>
       <c r="D8" s="4" t="s">
         <v>15</v>
@@ -1324,8 +1329,8 @@
       <c r="F8" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="G8" s="4">
-        <v>5</v>
+      <c r="G8" s="4" t="s">
+        <v>17</v>
       </c>
       <c r="H8" s="4"/>
       <c r="I8" s="4"/>
@@ -1341,14 +1346,14 @@
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A9" s="4" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B9" t="str">
         <f>IF(F9="","",IF(F9="end","test_end",F9&amp;"_"&amp;COUNTIF($F$2:F9,F9)))</f>
-        <v>run_normal_3</v>
+        <v>run_normal_2</v>
       </c>
       <c r="C9" s="3">
-        <v>3.2638888888888891E-2</v>
+        <v>1.7361111111111112E-2</v>
       </c>
       <c r="D9" s="4" t="s">
         <v>19</v>
@@ -1377,37 +1382,33 @@
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A10" s="4" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B10" t="str">
         <f>IF(F10="","",IF(F10="end","test_end",F10&amp;"_"&amp;COUNTIF($F$2:F10,F10)))</f>
-        <v>advanced_load_up_2</v>
+        <v>critical_peak_1</v>
       </c>
       <c r="C10" s="3">
-        <v>3.4027777777777775E-2</v>
+        <v>1.8749999999999999E-2</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="E10" t="str">
         <f t="shared" si="0"/>
         <v>cta</v>
       </c>
       <c r="F10" s="4" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="G10" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="H10" s="4">
-        <v>5</v>
-      </c>
-      <c r="I10" s="4" t="s">
-        <v>33</v>
-      </c>
+      <c r="H10" s="4"/>
+      <c r="I10" s="4"/>
       <c r="J10" s="2" t="str">
         <f>IFERROR(_xlfn.XLOOKUP(F10,'CTA Actions'!$A$2:$A$7,'CTA Actions'!$B$2:$B$7),"")</f>
-        <v>3|6</v>
+        <v>2|4</v>
       </c>
       <c r="K10" s="4"/>
       <c r="L10" s="4"/>
@@ -1417,14 +1418,14 @@
     </row>
     <row r="11" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A11" s="4" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B11" t="str">
         <f>IF(F11="","",IF(F11="end","test_end",F11&amp;"_"&amp;COUNTIF($F$2:F11,F11)))</f>
-        <v>run_normal_4</v>
+        <v>run_normal_3</v>
       </c>
       <c r="C11" s="3">
-        <v>3.5416666666666666E-2</v>
+        <v>2.1527777777777778E-2</v>
       </c>
       <c r="D11" s="4" t="s">
         <v>19</v>
@@ -1460,7 +1461,7 @@
         <v>test_end</v>
       </c>
       <c r="C12" s="3">
-        <v>5.5555555555555558E-3</v>
+        <v>2.2916666666666665E-2</v>
       </c>
       <c r="D12" s="4" t="s">
         <v>19</v>
@@ -9263,7 +9264,7 @@
     </row>
   </sheetData>
   <sheetProtection sheet="1" objects="1" scenarios="1"/>
-  <dataValidations xWindow="256" yWindow="493" count="9">
+  <dataValidations xWindow="561" yWindow="527" count="9">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid schedule value" error="Enter a value allowed for this schedule field." promptTitle="Action" prompt="The CTA-2045 command you want the run from the dropdown menu" sqref="F2:F336" xr:uid="{8634ECE3-E7CB-4581-95B1-4AB9629A7C09}">
       <formula1>"advanced_load_up,critical_peak,end,grid_emergency,load_up,run_normal,shed,water_draw"</formula1>
     </dataValidation>

</xml_diff>

<commit_message>
new schedule water draw test
</commit_message>
<xml_diff>
--- a/software/conformance_test_schedule_main.xlsx
+++ b/software/conformance_test_schedule_main.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pwrgra09-admin\Documents\myPythonFiles\Root\conformance_testing_team\software\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F58DDA62-622C-45E5-8AD5-73BABD2C484F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{16C8F3DD-D0D5-4BB2-ABB8-4D58616E10A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38190" yWindow="1170" windowWidth="25410" windowHeight="11295" xr2:uid="{C8C0DF4B-6D5B-4BD3-847D-4558E3821A3D}"/>
+    <workbookView xWindow="38400" yWindow="780" windowWidth="25410" windowHeight="11295" xr2:uid="{C8C0DF4B-6D5B-4BD3-847D-4558E3821A3D}"/>
   </bookViews>
   <sheets>
     <sheet name="conformance_test_schedule_main" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="37">
   <si>
     <t>enabled</t>
   </si>
@@ -134,9 +134,6 @@
   </si>
   <si>
     <t>Attemp Advanced Load up</t>
-  </si>
-  <si>
-    <t>100_wh</t>
   </si>
   <si>
     <t>Initial command</t>
@@ -1119,7 +1116,7 @@
       <c r="K2" s="4"/>
       <c r="L2" s="4"/>
       <c r="M2" s="4" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.25">
@@ -1128,38 +1125,36 @@
       </c>
       <c r="B3" t="str">
         <f>IF(F3="","",IF(F3="end","test_end",F3&amp;"_"&amp;COUNTIF($F$2:F3,F3)))</f>
-        <v>advanced_load_up_1</v>
+        <v>water_draw_1</v>
       </c>
       <c r="C3" s="3">
-        <v>2.0833333333333333E-3</v>
+        <v>6.9444444444444447E-4</v>
       </c>
       <c r="D3" s="4" t="s">
         <v>19</v>
       </c>
       <c r="E3" t="str">
         <f t="shared" ref="E3:E66" si="0">IF(F3="","",IF(F3="water_draw","water_draw",IF(F3="end","test","cta")))</f>
-        <v>cta</v>
+        <v>water_draw</v>
       </c>
       <c r="F3" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="G3" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="H3" s="4">
-        <v>5</v>
-      </c>
-      <c r="I3" s="4" t="s">
-        <v>33</v>
-      </c>
+        <v>36</v>
+      </c>
+      <c r="G3" s="4"/>
+      <c r="H3" s="4"/>
+      <c r="I3" s="4"/>
       <c r="J3" s="2" t="str">
         <f>IFERROR(_xlfn.XLOOKUP(F3,'CTA Actions'!$A$2:$A$7,'CTA Actions'!$B$2:$B$7),"")</f>
-        <v>3|6</v>
-      </c>
-      <c r="K3" s="4"/>
-      <c r="L3" s="4"/>
+        <v/>
+      </c>
+      <c r="K3" s="4">
+        <v>20</v>
+      </c>
+      <c r="L3" s="4">
+        <v>3</v>
+      </c>
       <c r="M3" s="4" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.25">
@@ -1195,7 +1190,7 @@
       <c r="K4" s="4"/>
       <c r="L4" s="4"/>
       <c r="M4" s="4" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.25">
@@ -1204,29 +1199,27 @@
       </c>
       <c r="B5" t="str">
         <f>IF(F5="","",IF(F5="end","test_end",F5&amp;"_"&amp;COUNTIF($F$2:F5,F5)))</f>
-        <v>load_up_1</v>
+        <v>test_end</v>
       </c>
       <c r="C5" s="3">
-        <v>5.5555555555555558E-3</v>
+        <v>6.2500000000000003E-3</v>
       </c>
       <c r="D5" s="4" t="s">
         <v>19</v>
       </c>
       <c r="E5" t="str">
         <f t="shared" si="0"/>
-        <v>cta</v>
+        <v>test</v>
       </c>
       <c r="F5" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="G5" s="4" t="s">
-        <v>17</v>
-      </c>
+        <v>20</v>
+      </c>
+      <c r="G5" s="4"/>
       <c r="H5" s="4"/>
       <c r="I5" s="4"/>
       <c r="J5" s="2" t="str">
         <f>IFERROR(_xlfn.XLOOKUP(F5,'CTA Actions'!$A$2:$A$7,'CTA Actions'!$B$2:$B$7),"")</f>
-        <v>3|6</v>
+        <v/>
       </c>
       <c r="K5" s="4"/>
       <c r="L5" s="4"/>
@@ -1236,7 +1229,7 @@
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B6" t="str">
         <f>IF(F6="","",IF(F6="end","test_end",F6&amp;"_"&amp;COUNTIF($F$2:F6,F6)))</f>
@@ -1272,11 +1265,11 @@
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B7" t="str">
         <f>IF(F7="","",IF(F7="end","test_end",F7&amp;"_"&amp;COUNTIF($F$2:F7,F7)))</f>
-        <v>water_draw_1</v>
+        <v>water_draw_2</v>
       </c>
       <c r="C7" s="3">
         <v>1.1111111111111112E-2</v>
@@ -1289,7 +1282,7 @@
         <v>water_draw</v>
       </c>
       <c r="F7" s="4" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="G7" s="4"/>
       <c r="H7" s="4"/>
@@ -1310,7 +1303,7 @@
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A8" s="4" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B8" t="str">
         <f>IF(F8="","",IF(F8="end","test_end",F8&amp;"_"&amp;COUNTIF($F$2:F8,F8)))</f>
@@ -1346,7 +1339,7 @@
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A9" s="4" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B9" t="str">
         <f>IF(F9="","",IF(F9="end","test_end",F9&amp;"_"&amp;COUNTIF($F$2:F9,F9)))</f>
@@ -1382,7 +1375,7 @@
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A10" s="4" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B10" t="str">
         <f>IF(F10="","",IF(F10="end","test_end",F10&amp;"_"&amp;COUNTIF($F$2:F10,F10)))</f>
@@ -1418,7 +1411,7 @@
     </row>
     <row r="11" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A11" s="4" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B11" t="str">
         <f>IF(F11="","",IF(F11="end","test_end",F11&amp;"_"&amp;COUNTIF($F$2:F11,F11)))</f>
@@ -1454,7 +1447,7 @@
     </row>
     <row r="12" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A12" s="4" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B12" t="str">
         <f>IF(F12="","",IF(F12="end","test_end",F12&amp;"_"&amp;COUNTIF($F$2:F12,F12)))</f>
@@ -9264,7 +9257,7 @@
     </row>
   </sheetData>
   <sheetProtection sheet="1" objects="1" scenarios="1"/>
-  <dataValidations xWindow="561" yWindow="527" count="9">
+  <dataValidations xWindow="167" yWindow="394" count="9">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid schedule value" error="Enter a value allowed for this schedule field." promptTitle="Action" prompt="The CTA-2045 command you want the run from the dropdown menu" sqref="F2:F336" xr:uid="{8634ECE3-E7CB-4581-95B1-4AB9629A7C09}">
       <formula1>"advanced_load_up,critical_peak,end,grid_emergency,load_up,run_normal,shed,water_draw"</formula1>
     </dataValidation>

</xml_diff>

<commit_message>
test new schedule on WH3
</commit_message>
<xml_diff>
--- a/software/conformance_test_schedule_main.xlsx
+++ b/software/conformance_test_schedule_main.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pwrgra09-admin\Documents\myPythonFiles\Root\conformance_testing_team\software\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5F94FD0C-78F9-46A0-B295-21E379A53F19}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EEEF1EB2-9D9C-4772-A019-595F1A5E507D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38400" yWindow="1170" windowWidth="25410" windowHeight="11295" xr2:uid="{C8C0DF4B-6D5B-4BD3-847D-4558E3821A3D}"/>
+    <workbookView xWindow="38190" yWindow="1560" windowWidth="25410" windowHeight="11295" xr2:uid="{C8C0DF4B-6D5B-4BD3-847D-4558E3821A3D}"/>
   </bookViews>
   <sheets>
     <sheet name="conformance_test_schedule_main" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="30">
   <si>
     <t>enabled</t>
   </si>
@@ -91,16 +91,10 @@
     <t>unknown</t>
   </si>
   <si>
-    <t>Return unit to normal</t>
-  </si>
-  <si>
     <t>recovery</t>
   </si>
   <si>
     <t>end</t>
-  </si>
-  <si>
-    <t>End recovery period</t>
   </si>
   <si>
     <t>event_duration_minutes</t>
@@ -127,25 +121,10 @@
     <t>1|0</t>
   </si>
   <si>
-    <t>Shed event</t>
+    <t>water_draw</t>
   </si>
   <si>
-    <t>Grid emergency event</t>
-  </si>
-  <si>
-    <t>Attemp Advanced Load up</t>
-  </si>
-  <si>
-    <t>Initial command</t>
-  </si>
-  <si>
-    <t>advanced load up</t>
-  </si>
-  <si>
-    <t>return to normal</t>
-  </si>
-  <si>
-    <t>water_draw</t>
+    <t>100_wh</t>
   </si>
 </sst>
 </file>
@@ -1062,7 +1041,7 @@
         <v>5</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="H1" s="1" t="s">
         <v>6</v>
@@ -1089,7 +1068,7 @@
       </c>
       <c r="B2" t="str">
         <f>IF(F2="","",IF(F2="end","test_end",F2&amp;"_"&amp;COUNTIF($F$2:F2,F2)))</f>
-        <v>shed_1</v>
+        <v>load_up_1</v>
       </c>
       <c r="C2" s="3">
         <v>0</v>
@@ -1102,7 +1081,7 @@
         <v>cta</v>
       </c>
       <c r="F2" s="4" t="s">
-        <v>27</v>
+        <v>13</v>
       </c>
       <c r="G2" s="4" t="s">
         <v>17</v>
@@ -1111,13 +1090,11 @@
       <c r="I2" s="4"/>
       <c r="J2" s="2" t="str">
         <f>IFERROR(_xlfn.XLOOKUP(F2,'CTA Actions'!$A$2:$A$7,'CTA Actions'!$B$2:$B$7),"")</f>
-        <v>2|4</v>
+        <v>3|6</v>
       </c>
       <c r="K2" s="4"/>
       <c r="L2" s="4"/>
-      <c r="M2" s="4" t="s">
-        <v>33</v>
-      </c>
+      <c r="M2" s="4"/>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A3" s="4" t="b">
@@ -1125,37 +1102,33 @@
       </c>
       <c r="B3" t="str">
         <f>IF(F3="","",IF(F3="end","test_end",F3&amp;"_"&amp;COUNTIF($F$2:F3,F3)))</f>
-        <v>water_draw_1</v>
+        <v>run_normal_1</v>
       </c>
       <c r="C3" s="3">
-        <v>6.9444444444444447E-4</v>
+        <v>4.8611111111111112E-3</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="E3" t="str">
         <f t="shared" ref="E3:E66" si="0">IF(F3="","",IF(F3="water_draw","water_draw",IF(F3="end","test","cta")))</f>
-        <v>water_draw</v>
+        <v>cta</v>
       </c>
       <c r="F3" s="4" t="s">
-        <v>36</v>
-      </c>
-      <c r="G3" s="4"/>
+        <v>16</v>
+      </c>
+      <c r="G3" s="4" t="s">
+        <v>17</v>
+      </c>
       <c r="H3" s="4"/>
       <c r="I3" s="4"/>
       <c r="J3" s="2" t="str">
         <f>IFERROR(_xlfn.XLOOKUP(F3,'CTA Actions'!$A$2:$A$7,'CTA Actions'!$B$2:$B$7),"")</f>
-        <v/>
-      </c>
-      <c r="K3" s="4">
-        <v>20</v>
-      </c>
-      <c r="L3" s="4">
-        <v>3</v>
-      </c>
-      <c r="M3" s="4" t="s">
-        <v>34</v>
-      </c>
+        <v>1|0</v>
+      </c>
+      <c r="K3" s="4"/>
+      <c r="L3" s="4"/>
+      <c r="M3" s="4"/>
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="b">
@@ -1163,20 +1136,20 @@
       </c>
       <c r="B4" t="str">
         <f>IF(F4="","",IF(F4="end","test_end",F4&amp;"_"&amp;COUNTIF($F$2:F4,F4)))</f>
-        <v>run_normal_1</v>
+        <v>shed_1</v>
       </c>
       <c r="C4" s="3">
-        <v>4.1666666666666666E-3</v>
+        <v>6.2500000000000003E-3</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="E4" t="str">
         <f t="shared" si="0"/>
         <v>cta</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>16</v>
+        <v>25</v>
       </c>
       <c r="G4" s="4" t="s">
         <v>17</v>
@@ -1185,13 +1158,11 @@
       <c r="I4" s="4"/>
       <c r="J4" s="2" t="str">
         <f>IFERROR(_xlfn.XLOOKUP(F4,'CTA Actions'!$A$2:$A$7,'CTA Actions'!$B$2:$B$7),"")</f>
-        <v>1|0</v>
+        <v>2|4</v>
       </c>
       <c r="K4" s="4"/>
       <c r="L4" s="4"/>
-      <c r="M4" s="4" t="s">
-        <v>35</v>
-      </c>
+      <c r="M4" s="4"/>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="b">
@@ -1199,20 +1170,20 @@
       </c>
       <c r="B5" t="str">
         <f>IF(F5="","",IF(F5="end","test_end",F5&amp;"_"&amp;COUNTIF($F$2:F5,F5)))</f>
-        <v>test_end</v>
+        <v>water_draw_1</v>
       </c>
       <c r="C5" s="3">
-        <v>6.2500000000000003E-3</v>
+        <v>8.3333333333333332E-3</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="E5" t="str">
         <f t="shared" si="0"/>
-        <v>test</v>
+        <v>water_draw</v>
       </c>
       <c r="F5" s="4" t="s">
-        <v>20</v>
+        <v>28</v>
       </c>
       <c r="G5" s="4"/>
       <c r="H5" s="4"/>
@@ -1221,32 +1192,34 @@
         <f>IFERROR(_xlfn.XLOOKUP(F5,'CTA Actions'!$A$2:$A$7,'CTA Actions'!$B$2:$B$7),"")</f>
         <v/>
       </c>
-      <c r="K5" s="4"/>
-      <c r="L5" s="4"/>
-      <c r="M5" s="4" t="s">
-        <v>18</v>
-      </c>
+      <c r="K5" s="4">
+        <v>9</v>
+      </c>
+      <c r="L5" s="4">
+        <v>3</v>
+      </c>
+      <c r="M5" s="4"/>
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B6" t="str">
         <f>IF(F6="","",IF(F6="end","test_end",F6&amp;"_"&amp;COUNTIF($F$2:F6,F6)))</f>
-        <v>shed_2</v>
+        <v>run_normal_2</v>
       </c>
       <c r="C6" s="3">
-        <v>9.7222222222222224E-3</v>
+        <v>1.1111111111111112E-2</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="E6" t="str">
         <f t="shared" si="0"/>
         <v>cta</v>
       </c>
       <c r="F6" s="4" t="s">
-        <v>27</v>
+        <v>16</v>
       </c>
       <c r="G6" s="4" t="s">
         <v>17</v>
@@ -1255,72 +1228,66 @@
       <c r="I6" s="4"/>
       <c r="J6" s="2" t="str">
         <f>IFERROR(_xlfn.XLOOKUP(F6,'CTA Actions'!$A$2:$A$7,'CTA Actions'!$B$2:$B$7),"")</f>
-        <v>2|4</v>
+        <v>1|0</v>
       </c>
       <c r="K6" s="4"/>
       <c r="L6" s="4"/>
-      <c r="M6" s="4" t="s">
-        <v>30</v>
-      </c>
+      <c r="M6" s="4"/>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B7" t="str">
         <f>IF(F7="","",IF(F7="end","test_end",F7&amp;"_"&amp;COUNTIF($F$2:F7,F7)))</f>
-        <v>water_draw_2</v>
+        <v>critical_peak_1</v>
       </c>
       <c r="C7" s="3">
-        <v>1.1111111111111112E-2</v>
+        <v>1.2500000000000001E-2</v>
       </c>
       <c r="D7" s="4" t="s">
         <v>15</v>
       </c>
       <c r="E7" t="str">
         <f t="shared" si="0"/>
-        <v>water_draw</v>
+        <v>cta</v>
       </c>
       <c r="F7" s="4" t="s">
-        <v>36</v>
-      </c>
-      <c r="G7" s="4"/>
+        <v>23</v>
+      </c>
+      <c r="G7" s="4" t="s">
+        <v>17</v>
+      </c>
       <c r="H7" s="4"/>
       <c r="I7" s="4"/>
       <c r="J7" s="2" t="str">
         <f>IFERROR(_xlfn.XLOOKUP(F7,'CTA Actions'!$A$2:$A$7,'CTA Actions'!$B$2:$B$7),"")</f>
-        <v/>
-      </c>
-      <c r="K7" s="4">
-        <v>9</v>
-      </c>
-      <c r="L7" s="4">
-        <v>3</v>
-      </c>
-      <c r="M7" s="4" t="s">
-        <v>18</v>
-      </c>
+        <v>2|4</v>
+      </c>
+      <c r="K7" s="4"/>
+      <c r="L7" s="4"/>
+      <c r="M7" s="4"/>
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A8" s="4" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B8" t="str">
         <f>IF(F8="","",IF(F8="end","test_end",F8&amp;"_"&amp;COUNTIF($F$2:F8,F8)))</f>
-        <v>grid_emergency_1</v>
+        <v>run_normal_3</v>
       </c>
       <c r="C8" s="3">
-        <v>1.4583333333333334E-2</v>
+        <v>1.6666666666666666E-2</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="E8" t="str">
         <f t="shared" si="0"/>
         <v>cta</v>
       </c>
       <c r="F8" s="4" t="s">
-        <v>26</v>
+        <v>16</v>
       </c>
       <c r="G8" s="4" t="s">
         <v>17</v>
@@ -1329,34 +1296,32 @@
       <c r="I8" s="4"/>
       <c r="J8" s="2" t="str">
         <f>IFERROR(_xlfn.XLOOKUP(F8,'CTA Actions'!$A$2:$A$7,'CTA Actions'!$B$2:$B$7),"")</f>
-        <v>2|4</v>
+        <v>1|0</v>
       </c>
       <c r="K8" s="4"/>
       <c r="L8" s="4"/>
-      <c r="M8" s="4" t="s">
-        <v>31</v>
-      </c>
+      <c r="M8" s="4"/>
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A9" s="4" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B9" t="str">
         <f>IF(F9="","",IF(F9="end","test_end",F9&amp;"_"&amp;COUNTIF($F$2:F9,F9)))</f>
-        <v>run_normal_2</v>
+        <v>grid_emergency_1</v>
       </c>
       <c r="C9" s="3">
-        <v>1.7361111111111112E-2</v>
+        <v>1.8055555555555554E-2</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="E9" t="str">
         <f t="shared" si="0"/>
         <v>cta</v>
       </c>
       <c r="F9" s="4" t="s">
-        <v>16</v>
+        <v>24</v>
       </c>
       <c r="G9" s="4" t="s">
         <v>17</v>
@@ -1365,34 +1330,32 @@
       <c r="I9" s="4"/>
       <c r="J9" s="2" t="str">
         <f>IFERROR(_xlfn.XLOOKUP(F9,'CTA Actions'!$A$2:$A$7,'CTA Actions'!$B$2:$B$7),"")</f>
-        <v>1|0</v>
+        <v>2|4</v>
       </c>
       <c r="K9" s="4"/>
       <c r="L9" s="4"/>
-      <c r="M9" s="4" t="s">
-        <v>18</v>
-      </c>
+      <c r="M9" s="4"/>
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A10" s="4" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B10" t="str">
         <f>IF(F10="","",IF(F10="end","test_end",F10&amp;"_"&amp;COUNTIF($F$2:F10,F10)))</f>
-        <v>critical_peak_1</v>
+        <v>run_normal_4</v>
       </c>
       <c r="C10" s="3">
-        <v>1.8749999999999999E-2</v>
+        <v>2.0833333333333332E-2</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="E10" t="str">
         <f t="shared" si="0"/>
         <v>cta</v>
       </c>
       <c r="F10" s="4" t="s">
-        <v>25</v>
+        <v>16</v>
       </c>
       <c r="G10" s="4" t="s">
         <v>17</v>
@@ -1401,34 +1364,32 @@
       <c r="I10" s="4"/>
       <c r="J10" s="2" t="str">
         <f>IFERROR(_xlfn.XLOOKUP(F10,'CTA Actions'!$A$2:$A$7,'CTA Actions'!$B$2:$B$7),"")</f>
-        <v>2|4</v>
+        <v>1|0</v>
       </c>
       <c r="K10" s="4"/>
       <c r="L10" s="4"/>
-      <c r="M10" s="4" t="s">
-        <v>32</v>
-      </c>
+      <c r="M10" s="4"/>
     </row>
     <row r="11" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A11" s="4" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B11" t="str">
         <f>IF(F11="","",IF(F11="end","test_end",F11&amp;"_"&amp;COUNTIF($F$2:F11,F11)))</f>
-        <v>run_normal_3</v>
+        <v>water_draw_2</v>
       </c>
       <c r="C11" s="3">
         <v>2.1527777777777778E-2</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="E11" t="str">
         <f t="shared" si="0"/>
-        <v>cta</v>
+        <v>water_draw</v>
       </c>
       <c r="F11" s="4" t="s">
-        <v>16</v>
+        <v>28</v>
       </c>
       <c r="G11" s="4" t="s">
         <v>17</v>
@@ -1437,83 +1398,109 @@
       <c r="I11" s="4"/>
       <c r="J11" s="2" t="str">
         <f>IFERROR(_xlfn.XLOOKUP(F11,'CTA Actions'!$A$2:$A$7,'CTA Actions'!$B$2:$B$7),"")</f>
-        <v>1|0</v>
-      </c>
-      <c r="K11" s="4"/>
-      <c r="L11" s="4"/>
-      <c r="M11" s="4" t="s">
-        <v>18</v>
-      </c>
+        <v/>
+      </c>
+      <c r="K11" s="4">
+        <v>6</v>
+      </c>
+      <c r="L11" s="4">
+        <v>3</v>
+      </c>
+      <c r="M11" s="4"/>
     </row>
     <row r="12" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A12" s="4" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B12" t="str">
         <f>IF(F12="","",IF(F12="end","test_end",F12&amp;"_"&amp;COUNTIF($F$2:F12,F12)))</f>
-        <v/>
+        <v>advanced_load_up_1</v>
       </c>
       <c r="C12" s="3">
-        <v>2.2916666666666665E-2</v>
+        <v>2.361111111111111E-2</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="E12" t="str">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="F12" s="4"/>
-      <c r="G12" s="4"/>
-      <c r="H12" s="4"/>
-      <c r="I12" s="4"/>
+        <v>cta</v>
+      </c>
+      <c r="F12" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="G12" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="H12" s="4">
+        <v>5</v>
+      </c>
+      <c r="I12" s="4" t="s">
+        <v>29</v>
+      </c>
       <c r="J12" s="2" t="str">
         <f>IFERROR(_xlfn.XLOOKUP(F12,'CTA Actions'!$A$2:$A$7,'CTA Actions'!$B$2:$B$7),"")</f>
-        <v/>
+        <v>3|6</v>
       </c>
       <c r="K12" s="4"/>
       <c r="L12" s="4"/>
-      <c r="M12" s="4" t="s">
-        <v>21</v>
-      </c>
+      <c r="M12" s="4"/>
     </row>
     <row r="13" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A13" s="4"/>
+      <c r="A13" s="4" t="b">
+        <v>1</v>
+      </c>
       <c r="B13" t="str">
         <f>IF(F13="","",IF(F13="end","test_end",F13&amp;"_"&amp;COUNTIF($F$2:F13,F13)))</f>
-        <v/>
-      </c>
-      <c r="C13" s="3"/>
-      <c r="D13" s="4"/>
+        <v>run_normal_5</v>
+      </c>
+      <c r="C13" s="3">
+        <v>2.7083333333333334E-2</v>
+      </c>
+      <c r="D13" s="4" t="s">
+        <v>18</v>
+      </c>
       <c r="E13" t="str">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="F13" s="4"/>
-      <c r="G13" s="4"/>
+        <v>cta</v>
+      </c>
+      <c r="F13" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G13" s="4" t="s">
+        <v>17</v>
+      </c>
       <c r="H13" s="4"/>
       <c r="I13" s="4"/>
       <c r="J13" s="2" t="str">
         <f>IFERROR(_xlfn.XLOOKUP(F13,'CTA Actions'!$A$2:$A$7,'CTA Actions'!$B$2:$B$7),"")</f>
-        <v/>
+        <v>1|0</v>
       </c>
       <c r="K13" s="4"/>
       <c r="L13" s="4"/>
       <c r="M13" s="4"/>
     </row>
     <row r="14" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A14" s="4"/>
+      <c r="A14" s="4" t="b">
+        <v>1</v>
+      </c>
       <c r="B14" t="str">
         <f>IF(F14="","",IF(F14="end","test_end",F14&amp;"_"&amp;COUNTIF($F$2:F14,F14)))</f>
-        <v/>
-      </c>
-      <c r="C14" s="3"/>
-      <c r="D14" s="4"/>
+        <v>test_end</v>
+      </c>
+      <c r="C14" s="3">
+        <v>2.7777777777777776E-2</v>
+      </c>
+      <c r="D14" s="4" t="s">
+        <v>18</v>
+      </c>
       <c r="E14" t="str">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="F14" s="4"/>
+        <v>test</v>
+      </c>
+      <c r="F14" s="4" t="s">
+        <v>19</v>
+      </c>
       <c r="G14" s="4"/>
       <c r="H14" s="4"/>
       <c r="I14" s="4"/>
@@ -9302,7 +9289,7 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>8</v>
@@ -9310,7 +9297,7 @@
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="B2" t="s">
         <v>14</v>
@@ -9318,18 +9305,18 @@
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="B3" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
+        <v>24</v>
+      </c>
+      <c r="B4" t="s">
         <v>26</v>
-      </c>
-      <c r="B4" t="s">
-        <v>28</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
@@ -9345,15 +9332,15 @@
         <v>16</v>
       </c>
       <c r="B6" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="B7" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix water draw argument
</commit_message>
<xml_diff>
--- a/software/conformance_test_schedule_main.xlsx
+++ b/software/conformance_test_schedule_main.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pwrgra09-admin\Documents\myPythonFiles\Root\conformance_testing_team\software\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EEEF1EB2-9D9C-4772-A019-595F1A5E507D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{929A2AB3-0AE2-4767-BA09-33AD3170E35C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="38190" yWindow="1560" windowWidth="25410" windowHeight="11295" xr2:uid="{C8C0DF4B-6D5B-4BD3-847D-4558E3821A3D}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="30">
   <si>
     <t>enabled</t>
   </si>
@@ -1391,9 +1391,7 @@
       <c r="F11" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="G11" s="4" t="s">
-        <v>17</v>
-      </c>
+      <c r="G11" s="4"/>
       <c r="H11" s="4"/>
       <c r="I11" s="4"/>
       <c r="J11" s="2" t="str">
@@ -9242,7 +9240,7 @@
     </row>
   </sheetData>
   <sheetProtection sheet="1" objects="1" scenarios="1"/>
-  <dataValidations xWindow="167" yWindow="394" count="9">
+  <dataValidations disablePrompts="1" xWindow="167" yWindow="394" count="9">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid schedule value" error="Enter a value allowed for this schedule field." promptTitle="Action" prompt="The CTA-2045 command you want the run from the dropdown menu" sqref="F2:F336" xr:uid="{8634ECE3-E7CB-4581-95B1-4AB9629A7C09}">
       <formula1>"advanced_load_up,critical_peak,end,grid_emergency,load_up,run_normal,shed,water_draw"</formula1>
     </dataValidation>

</xml_diff>

<commit_message>
updated data parser to put csv files nested in WH-n folder and update schedule
</commit_message>
<xml_diff>
--- a/software/conformance_test_schedule_main.xlsx
+++ b/software/conformance_test_schedule_main.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pwrgra09-admin\Documents\myPythonFiles\Root\conformance_testing_team\software\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{929A2AB3-0AE2-4767-BA09-33AD3170E35C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7599DEE3-CAB9-40AF-B9D5-FDB2C67FD32A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38190" yWindow="1560" windowWidth="25410" windowHeight="11295" xr2:uid="{C8C0DF4B-6D5B-4BD3-847D-4558E3821A3D}"/>
+    <workbookView xWindow="38280" yWindow="-120" windowWidth="25440" windowHeight="15270" xr2:uid="{C8C0DF4B-6D5B-4BD3-847D-4558E3821A3D}"/>
   </bookViews>
   <sheets>
     <sheet name="conformance_test_schedule_main" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="29">
   <si>
     <t>enabled</t>
   </si>
@@ -122,9 +122,6 @@
   </si>
   <si>
     <t>water_draw</t>
-  </si>
-  <si>
-    <t>100_wh</t>
   </si>
 </sst>
 </file>
@@ -1105,10 +1102,10 @@
         <v>run_normal_1</v>
       </c>
       <c r="C3" s="3">
-        <v>4.8611111111111112E-3</v>
+        <v>6.25E-2</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="E3" t="str">
         <f t="shared" ref="E3:E66" si="0">IF(F3="","",IF(F3="water_draw","water_draw",IF(F3="end","test","cta")))</f>
@@ -1136,32 +1133,34 @@
       </c>
       <c r="B4" t="str">
         <f>IF(F4="","",IF(F4="end","test_end",F4&amp;"_"&amp;COUNTIF($F$2:F4,F4)))</f>
-        <v>shed_1</v>
+        <v>water_draw_1</v>
       </c>
       <c r="C4" s="3">
-        <v>6.2500000000000003E-3</v>
+        <v>8.3333333333333329E-2</v>
       </c>
       <c r="D4" s="4" t="s">
         <v>15</v>
       </c>
       <c r="E4" t="str">
         <f t="shared" si="0"/>
-        <v>cta</v>
+        <v>water_draw</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="G4" s="4" t="s">
-        <v>17</v>
-      </c>
+        <v>28</v>
+      </c>
+      <c r="G4" s="4"/>
       <c r="H4" s="4"/>
       <c r="I4" s="4"/>
       <c r="J4" s="2" t="str">
         <f>IFERROR(_xlfn.XLOOKUP(F4,'CTA Actions'!$A$2:$A$7,'CTA Actions'!$B$2:$B$7),"")</f>
-        <v>2|4</v>
-      </c>
-      <c r="K4" s="4"/>
-      <c r="L4" s="4"/>
+        <v/>
+      </c>
+      <c r="K4" s="4">
+        <v>15</v>
+      </c>
+      <c r="L4" s="4">
+        <v>3</v>
+      </c>
       <c r="M4" s="4"/>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.25">
@@ -1170,10 +1169,10 @@
       </c>
       <c r="B5" t="str">
         <f>IF(F5="","",IF(F5="end","test_end",F5&amp;"_"&amp;COUNTIF($F$2:F5,F5)))</f>
-        <v>water_draw_1</v>
+        <v>water_draw_2</v>
       </c>
       <c r="C5" s="3">
-        <v>8.3333333333333332E-3</v>
+        <v>0.10416666666666667</v>
       </c>
       <c r="D5" s="4" t="s">
         <v>15</v>
@@ -1193,7 +1192,7 @@
         <v/>
       </c>
       <c r="K5" s="4">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="L5" s="4">
         <v>3</v>
@@ -1206,32 +1205,34 @@
       </c>
       <c r="B6" t="str">
         <f>IF(F6="","",IF(F6="end","test_end",F6&amp;"_"&amp;COUNTIF($F$2:F6,F6)))</f>
-        <v>run_normal_2</v>
+        <v>water_draw_3</v>
       </c>
       <c r="C6" s="3">
-        <v>1.1111111111111112E-2</v>
+        <v>0.15277777777777779</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="E6" t="str">
         <f t="shared" si="0"/>
-        <v>cta</v>
+        <v>water_draw</v>
       </c>
       <c r="F6" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="G6" s="4" t="s">
-        <v>17</v>
-      </c>
+        <v>28</v>
+      </c>
+      <c r="G6" s="4"/>
       <c r="H6" s="4"/>
       <c r="I6" s="4"/>
       <c r="J6" s="2" t="str">
         <f>IFERROR(_xlfn.XLOOKUP(F6,'CTA Actions'!$A$2:$A$7,'CTA Actions'!$B$2:$B$7),"")</f>
-        <v>1|0</v>
-      </c>
-      <c r="K6" s="4"/>
-      <c r="L6" s="4"/>
+        <v/>
+      </c>
+      <c r="K6" s="4">
+        <v>9</v>
+      </c>
+      <c r="L6" s="4">
+        <v>3</v>
+      </c>
       <c r="M6" s="4"/>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.25">
@@ -1240,20 +1241,20 @@
       </c>
       <c r="B7" t="str">
         <f>IF(F7="","",IF(F7="end","test_end",F7&amp;"_"&amp;COUNTIF($F$2:F7,F7)))</f>
-        <v>critical_peak_1</v>
+        <v>load_up_2</v>
       </c>
       <c r="C7" s="3">
-        <v>1.2500000000000001E-2</v>
+        <v>0.19444444444444445</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="E7" t="str">
         <f t="shared" si="0"/>
         <v>cta</v>
       </c>
       <c r="F7" s="4" t="s">
-        <v>23</v>
+        <v>13</v>
       </c>
       <c r="G7" s="4" t="s">
         <v>17</v>
@@ -1262,7 +1263,7 @@
       <c r="I7" s="4"/>
       <c r="J7" s="2" t="str">
         <f>IFERROR(_xlfn.XLOOKUP(F7,'CTA Actions'!$A$2:$A$7,'CTA Actions'!$B$2:$B$7),"")</f>
-        <v>2|4</v>
+        <v>3|6</v>
       </c>
       <c r="K7" s="4"/>
       <c r="L7" s="4"/>
@@ -1274,10 +1275,10 @@
       </c>
       <c r="B8" t="str">
         <f>IF(F8="","",IF(F8="end","test_end",F8&amp;"_"&amp;COUNTIF($F$2:F8,F8)))</f>
-        <v>run_normal_3</v>
+        <v>run_normal_2</v>
       </c>
       <c r="C8" s="3">
-        <v>1.6666666666666666E-2</v>
+        <v>0.2361111111111111</v>
       </c>
       <c r="D8" s="4" t="s">
         <v>18</v>
@@ -1308,89 +1309,69 @@
       </c>
       <c r="B9" t="str">
         <f>IF(F9="","",IF(F9="end","test_end",F9&amp;"_"&amp;COUNTIF($F$2:F9,F9)))</f>
-        <v>grid_emergency_1</v>
+        <v>test_end</v>
       </c>
       <c r="C9" s="3">
-        <v>1.8055555555555554E-2</v>
+        <v>0.25</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="E9" t="str">
         <f t="shared" si="0"/>
-        <v>cta</v>
+        <v>test</v>
       </c>
       <c r="F9" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="G9" s="4" t="s">
-        <v>17</v>
-      </c>
+        <v>19</v>
+      </c>
+      <c r="G9" s="4"/>
       <c r="H9" s="4"/>
       <c r="I9" s="4"/>
       <c r="J9" s="2" t="str">
         <f>IFERROR(_xlfn.XLOOKUP(F9,'CTA Actions'!$A$2:$A$7,'CTA Actions'!$B$2:$B$7),"")</f>
-        <v>2|4</v>
+        <v/>
       </c>
       <c r="K9" s="4"/>
       <c r="L9" s="4"/>
       <c r="M9" s="4"/>
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A10" s="4" t="b">
-        <v>1</v>
-      </c>
+      <c r="A10" s="4"/>
       <c r="B10" t="str">
         <f>IF(F10="","",IF(F10="end","test_end",F10&amp;"_"&amp;COUNTIF($F$2:F10,F10)))</f>
-        <v>run_normal_4</v>
-      </c>
-      <c r="C10" s="3">
-        <v>2.0833333333333332E-2</v>
-      </c>
-      <c r="D10" s="4" t="s">
-        <v>18</v>
-      </c>
+        <v/>
+      </c>
+      <c r="C10" s="3"/>
+      <c r="D10" s="4"/>
       <c r="E10" t="str">
         <f t="shared" si="0"/>
-        <v>cta</v>
-      </c>
-      <c r="F10" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="G10" s="4" t="s">
-        <v>17</v>
-      </c>
+        <v/>
+      </c>
+      <c r="F10" s="4"/>
+      <c r="G10" s="4"/>
       <c r="H10" s="4"/>
       <c r="I10" s="4"/>
       <c r="J10" s="2" t="str">
         <f>IFERROR(_xlfn.XLOOKUP(F10,'CTA Actions'!$A$2:$A$7,'CTA Actions'!$B$2:$B$7),"")</f>
-        <v>1|0</v>
+        <v/>
       </c>
       <c r="K10" s="4"/>
       <c r="L10" s="4"/>
       <c r="M10" s="4"/>
     </row>
     <row r="11" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A11" s="4" t="b">
-        <v>1</v>
-      </c>
+      <c r="A11" s="4"/>
       <c r="B11" t="str">
         <f>IF(F11="","",IF(F11="end","test_end",F11&amp;"_"&amp;COUNTIF($F$2:F11,F11)))</f>
-        <v>water_draw_2</v>
-      </c>
-      <c r="C11" s="3">
-        <v>2.1527777777777778E-2</v>
-      </c>
-      <c r="D11" s="4" t="s">
-        <v>15</v>
-      </c>
+        <v/>
+      </c>
+      <c r="C11" s="3"/>
+      <c r="D11" s="4"/>
       <c r="E11" t="str">
         <f t="shared" si="0"/>
-        <v>water_draw</v>
-      </c>
-      <c r="F11" s="4" t="s">
-        <v>28</v>
-      </c>
+        <v/>
+      </c>
+      <c r="F11" s="4"/>
       <c r="G11" s="4"/>
       <c r="H11" s="4"/>
       <c r="I11" s="4"/>
@@ -1398,107 +1379,71 @@
         <f>IFERROR(_xlfn.XLOOKUP(F11,'CTA Actions'!$A$2:$A$7,'CTA Actions'!$B$2:$B$7),"")</f>
         <v/>
       </c>
-      <c r="K11" s="4">
-        <v>6</v>
-      </c>
-      <c r="L11" s="4">
-        <v>3</v>
-      </c>
+      <c r="K11" s="4"/>
+      <c r="L11" s="4"/>
       <c r="M11" s="4"/>
     </row>
     <row r="12" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A12" s="4" t="b">
-        <v>1</v>
-      </c>
+      <c r="A12" s="4"/>
       <c r="B12" t="str">
         <f>IF(F12="","",IF(F12="end","test_end",F12&amp;"_"&amp;COUNTIF($F$2:F12,F12)))</f>
-        <v>advanced_load_up_1</v>
-      </c>
-      <c r="C12" s="3">
-        <v>2.361111111111111E-2</v>
-      </c>
-      <c r="D12" s="4" t="s">
-        <v>15</v>
-      </c>
+        <v/>
+      </c>
+      <c r="C12" s="3"/>
+      <c r="D12" s="4"/>
       <c r="E12" t="str">
         <f t="shared" si="0"/>
-        <v>cta</v>
-      </c>
-      <c r="F12" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="G12" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="H12" s="4">
-        <v>5</v>
-      </c>
-      <c r="I12" s="4" t="s">
-        <v>29</v>
-      </c>
+        <v/>
+      </c>
+      <c r="F12" s="4"/>
+      <c r="G12" s="4"/>
+      <c r="H12" s="4"/>
+      <c r="I12" s="4"/>
       <c r="J12" s="2" t="str">
         <f>IFERROR(_xlfn.XLOOKUP(F12,'CTA Actions'!$A$2:$A$7,'CTA Actions'!$B$2:$B$7),"")</f>
-        <v>3|6</v>
+        <v/>
       </c>
       <c r="K12" s="4"/>
       <c r="L12" s="4"/>
       <c r="M12" s="4"/>
     </row>
     <row r="13" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A13" s="4" t="b">
-        <v>1</v>
-      </c>
+      <c r="A13" s="4"/>
       <c r="B13" t="str">
         <f>IF(F13="","",IF(F13="end","test_end",F13&amp;"_"&amp;COUNTIF($F$2:F13,F13)))</f>
-        <v>run_normal_5</v>
-      </c>
-      <c r="C13" s="3">
-        <v>2.7083333333333334E-2</v>
-      </c>
-      <c r="D13" s="4" t="s">
-        <v>18</v>
-      </c>
+        <v/>
+      </c>
+      <c r="C13" s="3"/>
+      <c r="D13" s="4"/>
       <c r="E13" t="str">
         <f t="shared" si="0"/>
-        <v>cta</v>
-      </c>
-      <c r="F13" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="G13" s="4" t="s">
-        <v>17</v>
-      </c>
+        <v/>
+      </c>
+      <c r="F13" s="4"/>
+      <c r="G13" s="4"/>
       <c r="H13" s="4"/>
       <c r="I13" s="4"/>
       <c r="J13" s="2" t="str">
         <f>IFERROR(_xlfn.XLOOKUP(F13,'CTA Actions'!$A$2:$A$7,'CTA Actions'!$B$2:$B$7),"")</f>
-        <v>1|0</v>
+        <v/>
       </c>
       <c r="K13" s="4"/>
       <c r="L13" s="4"/>
       <c r="M13" s="4"/>
     </row>
     <row r="14" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A14" s="4" t="b">
-        <v>1</v>
-      </c>
+      <c r="A14" s="4"/>
       <c r="B14" t="str">
         <f>IF(F14="","",IF(F14="end","test_end",F14&amp;"_"&amp;COUNTIF($F$2:F14,F14)))</f>
-        <v>test_end</v>
-      </c>
-      <c r="C14" s="3">
-        <v>2.7777777777777776E-2</v>
-      </c>
-      <c r="D14" s="4" t="s">
-        <v>18</v>
-      </c>
+        <v/>
+      </c>
+      <c r="C14" s="3"/>
+      <c r="D14" s="4"/>
       <c r="E14" t="str">
         <f t="shared" si="0"/>
-        <v>test</v>
-      </c>
-      <c r="F14" s="4" t="s">
-        <v>19</v>
-      </c>
+        <v/>
+      </c>
+      <c r="F14" s="4"/>
       <c r="G14" s="4"/>
       <c r="H14" s="4"/>
       <c r="I14" s="4"/>

</xml_diff>

<commit_message>
new test for duration of load up
</commit_message>
<xml_diff>
--- a/software/conformance_test_schedule_main.xlsx
+++ b/software/conformance_test_schedule_main.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pwrgra09-admin\Documents\myPythonFiles\Root\conformance_testing_team\software\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7599DEE3-CAB9-40AF-B9D5-FDB2C67FD32A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{43A3FB3F-6E6C-4C31-AF2A-5ABF998D4C80}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="38280" yWindow="-120" windowWidth="25440" windowHeight="15270" xr2:uid="{C8C0DF4B-6D5B-4BD3-847D-4558E3821A3D}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="29">
   <si>
     <t>enabled</t>
   </si>
@@ -1080,8 +1080,8 @@
       <c r="F2" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="G2" s="4" t="s">
-        <v>17</v>
+      <c r="G2" s="4">
+        <v>20</v>
       </c>
       <c r="H2" s="4"/>
       <c r="I2" s="4"/>
@@ -1102,7 +1102,7 @@
         <v>run_normal_1</v>
       </c>
       <c r="C3" s="3">
-        <v>6.25E-2</v>
+        <v>1.7361111111111112E-2</v>
       </c>
       <c r="D3" s="4" t="s">
         <v>15</v>
@@ -1133,20 +1133,20 @@
       </c>
       <c r="B4" t="str">
         <f>IF(F4="","",IF(F4="end","test_end",F4&amp;"_"&amp;COUNTIF($F$2:F4,F4)))</f>
-        <v>water_draw_1</v>
+        <v>test_end</v>
       </c>
       <c r="C4" s="3">
-        <v>8.3333333333333329E-2</v>
+        <v>1.8749999999999999E-2</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="E4" t="str">
         <f t="shared" si="0"/>
-        <v>water_draw</v>
+        <v>test</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>28</v>
+        <v>19</v>
       </c>
       <c r="G4" s="4"/>
       <c r="H4" s="4"/>
@@ -1155,21 +1155,17 @@
         <f>IFERROR(_xlfn.XLOOKUP(F4,'CTA Actions'!$A$2:$A$7,'CTA Actions'!$B$2:$B$7),"")</f>
         <v/>
       </c>
-      <c r="K4" s="4">
-        <v>15</v>
-      </c>
-      <c r="L4" s="4">
-        <v>3</v>
-      </c>
+      <c r="K4" s="4"/>
+      <c r="L4" s="4"/>
       <c r="M4" s="4"/>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B5" t="str">
         <f>IF(F5="","",IF(F5="end","test_end",F5&amp;"_"&amp;COUNTIF($F$2:F5,F5)))</f>
-        <v>water_draw_2</v>
+        <v>water_draw_1</v>
       </c>
       <c r="C5" s="3">
         <v>0.10416666666666667</v>
@@ -1201,11 +1197,11 @@
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B6" t="str">
         <f>IF(F6="","",IF(F6="end","test_end",F6&amp;"_"&amp;COUNTIF($F$2:F6,F6)))</f>
-        <v>water_draw_3</v>
+        <v>water_draw_2</v>
       </c>
       <c r="C6" s="3">
         <v>0.15277777777777779</v>
@@ -1237,7 +1233,7 @@
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B7" t="str">
         <f>IF(F7="","",IF(F7="end","test_end",F7&amp;"_"&amp;COUNTIF($F$2:F7,F7)))</f>
@@ -1271,7 +1267,7 @@
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A8" s="4" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B8" t="str">
         <f>IF(F8="","",IF(F8="end","test_end",F8&amp;"_"&amp;COUNTIF($F$2:F8,F8)))</f>
@@ -1305,11 +1301,11 @@
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A9" s="4" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B9" t="str">
         <f>IF(F9="","",IF(F9="end","test_end",F9&amp;"_"&amp;COUNTIF($F$2:F9,F9)))</f>
-        <v>test_end</v>
+        <v/>
       </c>
       <c r="C9" s="3">
         <v>0.25</v>
@@ -1319,11 +1315,9 @@
       </c>
       <c r="E9" t="str">
         <f t="shared" si="0"/>
-        <v>test</v>
-      </c>
-      <c r="F9" s="4" t="s">
-        <v>19</v>
-      </c>
+        <v/>
+      </c>
+      <c r="F9" s="4"/>
       <c r="G9" s="4"/>
       <c r="H9" s="4"/>
       <c r="I9" s="4"/>
@@ -9185,7 +9179,7 @@
     </row>
   </sheetData>
   <sheetProtection sheet="1" objects="1" scenarios="1"/>
-  <dataValidations disablePrompts="1" xWindow="167" yWindow="394" count="9">
+  <dataValidations xWindow="167" yWindow="394" count="9">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid schedule value" error="Enter a value allowed for this schedule field." promptTitle="Action" prompt="The CTA-2045 command you want the run from the dropdown menu" sqref="F2:F336" xr:uid="{8634ECE3-E7CB-4581-95B1-4AB9629A7C09}">
       <formula1>"advanced_load_up,critical_peak,end,grid_emergency,load_up,run_normal,shed,water_draw"</formula1>
     </dataValidation>

</xml_diff>

<commit_message>
update to test unknown schedule with outside comm heartbeat
</commit_message>
<xml_diff>
--- a/software/conformance_test_schedule_main.xlsx
+++ b/software/conformance_test_schedule_main.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pwrgra09-admin\Documents\myPythonFiles\Root\conformance_testing_team\software\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{43A3FB3F-6E6C-4C31-AF2A-5ABF998D4C80}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{988E2885-8108-4626-9B94-F89391C88666}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38280" yWindow="-120" windowWidth="25440" windowHeight="15270" xr2:uid="{C8C0DF4B-6D5B-4BD3-847D-4558E3821A3D}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="15720" xr2:uid="{C8C0DF4B-6D5B-4BD3-847D-4558E3821A3D}"/>
   </bookViews>
   <sheets>
     <sheet name="conformance_test_schedule_main" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="29">
   <si>
     <t>enabled</t>
   </si>
@@ -1080,8 +1080,8 @@
       <c r="F2" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="G2" s="4">
-        <v>20</v>
+      <c r="G2" s="4" t="s">
+        <v>17</v>
       </c>
       <c r="H2" s="4"/>
       <c r="I2" s="4"/>
@@ -1102,7 +1102,7 @@
         <v>run_normal_1</v>
       </c>
       <c r="C3" s="3">
-        <v>1.7361111111111112E-2</v>
+        <v>2.0833333333333332E-2</v>
       </c>
       <c r="D3" s="4" t="s">
         <v>15</v>
@@ -1136,7 +1136,7 @@
         <v>test_end</v>
       </c>
       <c r="C4" s="3">
-        <v>1.8749999999999999E-2</v>
+        <v>2.1527777777777778E-2</v>
       </c>
       <c r="D4" s="4" t="s">
         <v>18</v>

</xml_diff>

<commit_message>
updated the schedule to retest LU-Normal-Recovery
</commit_message>
<xml_diff>
--- a/software/conformance_test_schedule_main.xlsx
+++ b/software/conformance_test_schedule_main.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pwrgra09-admin\Documents\myPythonFiles\Root\conformance_testing_team\software\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{988E2885-8108-4626-9B94-F89391C88666}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3BCB132B-E603-45D4-917D-A26EFC2BA1FA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="15720" xr2:uid="{C8C0DF4B-6D5B-4BD3-847D-4558E3821A3D}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="29">
   <si>
     <t>enabled</t>
   </si>
@@ -1102,7 +1102,7 @@
         <v>run_normal_1</v>
       </c>
       <c r="C3" s="3">
-        <v>2.0833333333333332E-2</v>
+        <v>6.25E-2</v>
       </c>
       <c r="D3" s="4" t="s">
         <v>15</v>
@@ -1133,20 +1133,20 @@
       </c>
       <c r="B4" t="str">
         <f>IF(F4="","",IF(F4="end","test_end",F4&amp;"_"&amp;COUNTIF($F$2:F4,F4)))</f>
-        <v>test_end</v>
+        <v>water_draw_1</v>
       </c>
       <c r="C4" s="3">
-        <v>2.1527777777777778E-2</v>
+        <v>8.3333333333333329E-2</v>
       </c>
       <c r="D4" s="4" t="s">
         <v>18</v>
       </c>
       <c r="E4" t="str">
         <f t="shared" si="0"/>
-        <v>test</v>
+        <v>water_draw</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>19</v>
+        <v>28</v>
       </c>
       <c r="G4" s="4"/>
       <c r="H4" s="4"/>
@@ -1155,17 +1155,21 @@
         <f>IFERROR(_xlfn.XLOOKUP(F4,'CTA Actions'!$A$2:$A$7,'CTA Actions'!$B$2:$B$7),"")</f>
         <v/>
       </c>
-      <c r="K4" s="4"/>
-      <c r="L4" s="4"/>
+      <c r="K4" s="4">
+        <v>15</v>
+      </c>
+      <c r="L4" s="4">
+        <v>3</v>
+      </c>
       <c r="M4" s="4"/>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B5" t="str">
         <f>IF(F5="","",IF(F5="end","test_end",F5&amp;"_"&amp;COUNTIF($F$2:F5,F5)))</f>
-        <v>water_draw_1</v>
+        <v>water_draw_2</v>
       </c>
       <c r="C5" s="3">
         <v>0.10416666666666667</v>
@@ -1197,11 +1201,11 @@
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B6" t="str">
         <f>IF(F6="","",IF(F6="end","test_end",F6&amp;"_"&amp;COUNTIF($F$2:F6,F6)))</f>
-        <v>water_draw_2</v>
+        <v>water_draw_3</v>
       </c>
       <c r="C6" s="3">
         <v>0.15277777777777779</v>
@@ -1233,7 +1237,7 @@
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B7" t="str">
         <f>IF(F7="","",IF(F7="end","test_end",F7&amp;"_"&amp;COUNTIF($F$2:F7,F7)))</f>
@@ -1267,7 +1271,7 @@
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A8" s="4" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B8" t="str">
         <f>IF(F8="","",IF(F8="end","test_end",F8&amp;"_"&amp;COUNTIF($F$2:F8,F8)))</f>
@@ -1301,11 +1305,11 @@
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A9" s="4" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B9" t="str">
         <f>IF(F9="","",IF(F9="end","test_end",F9&amp;"_"&amp;COUNTIF($F$2:F9,F9)))</f>
-        <v/>
+        <v>test_end</v>
       </c>
       <c r="C9" s="3">
         <v>0.25</v>
@@ -1315,9 +1319,11 @@
       </c>
       <c r="E9" t="str">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="F9" s="4"/>
+        <v>test</v>
+      </c>
+      <c r="F9" s="4" t="s">
+        <v>19</v>
+      </c>
       <c r="G9" s="4"/>
       <c r="H9" s="4"/>
       <c r="I9" s="4"/>

</xml_diff>

<commit_message>
updating for new schedule LU-CPE-Recovery and changing the power recording sensativity
</commit_message>
<xml_diff>
--- a/software/conformance_test_schedule_main.xlsx
+++ b/software/conformance_test_schedule_main.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pwrgra09-admin\Documents\myPythonFiles\Root\conformance_testing_team\software\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B99440AA-B1CE-4301-B260-C43F4679AA03}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6C411AE8-F195-4E9D-8720-0F694B194EFD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="15720" xr2:uid="{C8C0DF4B-6D5B-4BD3-847D-4558E3821A3D}"/>
+    <workbookView xWindow="8550" yWindow="1665" windowWidth="21600" windowHeight="11295" xr2:uid="{C8C0DF4B-6D5B-4BD3-847D-4558E3821A3D}"/>
   </bookViews>
   <sheets>
     <sheet name="conformance_test_schedule_main" sheetId="1" r:id="rId1"/>
@@ -1099,7 +1099,7 @@
       </c>
       <c r="B3" t="str">
         <f>IF(F3="","",IF(F3="end","test_end",F3&amp;"_"&amp;COUNTIF($F$2:F3,F3)))</f>
-        <v>shed_1</v>
+        <v>critical_peak_1</v>
       </c>
       <c r="C3" s="3">
         <v>6.25E-2</v>
@@ -1112,7 +1112,7 @@
         <v>cta</v>
       </c>
       <c r="F3" s="4" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="G3" s="4" t="s">
         <v>17</v>

</xml_diff>

<commit_message>
updated schedule and recording of operational state in the report script
</commit_message>
<xml_diff>
--- a/software/conformance_test_schedule_main.xlsx
+++ b/software/conformance_test_schedule_main.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pwrgra09-admin\Documents\myPythonFiles\Root\conformance_testing_team\software\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6C411AE8-F195-4E9D-8720-0F694B194EFD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7B73ABD0-A881-4686-9221-943CE5A4F223}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="8550" yWindow="1665" windowWidth="21600" windowHeight="11295" xr2:uid="{C8C0DF4B-6D5B-4BD3-847D-4558E3821A3D}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="15720" xr2:uid="{C8C0DF4B-6D5B-4BD3-847D-4558E3821A3D}"/>
   </bookViews>
   <sheets>
     <sheet name="conformance_test_schedule_main" sheetId="1" r:id="rId1"/>
@@ -1099,7 +1099,7 @@
       </c>
       <c r="B3" t="str">
         <f>IF(F3="","",IF(F3="end","test_end",F3&amp;"_"&amp;COUNTIF($F$2:F3,F3)))</f>
-        <v>critical_peak_1</v>
+        <v>grid_emergency_1</v>
       </c>
       <c r="C3" s="3">
         <v>6.25E-2</v>
@@ -1112,7 +1112,7 @@
         <v>cta</v>
       </c>
       <c r="F3" s="4" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="G3" s="4" t="s">
         <v>17</v>

</xml_diff>

<commit_message>
removed unknown duration value and installed max duration value
</commit_message>
<xml_diff>
--- a/software/conformance_test_schedule_main.xlsx
+++ b/software/conformance_test_schedule_main.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pwrgra09-admin\Documents\myPythonFiles\Root\conformance_testing_team\software\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7B73ABD0-A881-4686-9221-943CE5A4F223}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C06BEF90-A371-418C-83A5-E14FD0B228EE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="15720" xr2:uid="{C8C0DF4B-6D5B-4BD3-847D-4558E3821A3D}"/>
   </bookViews>
@@ -88,9 +88,6 @@
     <t>run_normal</t>
   </si>
   <si>
-    <t>unknown</t>
-  </si>
-  <si>
     <t>recovery</t>
   </si>
   <si>
@@ -122,6 +119,9 @@
   </si>
   <si>
     <t>water_draw</t>
+  </si>
+  <si>
+    <t>max</t>
   </si>
 </sst>
 </file>
@@ -1038,7 +1038,7 @@
         <v>5</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="H1" s="1" t="s">
         <v>6</v>
@@ -1081,7 +1081,7 @@
         <v>13</v>
       </c>
       <c r="G2" s="4" t="s">
-        <v>17</v>
+        <v>28</v>
       </c>
       <c r="H2" s="4"/>
       <c r="I2" s="4"/>
@@ -1112,10 +1112,10 @@
         <v>cta</v>
       </c>
       <c r="F3" s="4" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="G3" s="4" t="s">
-        <v>17</v>
+        <v>28</v>
       </c>
       <c r="H3" s="4"/>
       <c r="I3" s="4"/>
@@ -1139,14 +1139,14 @@
         <v>8.3333333333333329E-2</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="E4" t="str">
         <f t="shared" si="0"/>
         <v>water_draw</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="G4" s="4"/>
       <c r="H4" s="4"/>
@@ -1182,7 +1182,7 @@
         <v>water_draw</v>
       </c>
       <c r="F5" s="4" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="G5" s="4"/>
       <c r="H5" s="4"/>
@@ -1218,7 +1218,7 @@
         <v>water_draw</v>
       </c>
       <c r="F6" s="4" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="G6" s="4"/>
       <c r="H6" s="4"/>
@@ -1247,7 +1247,7 @@
         <v>0.19444444444444445</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="E7" t="str">
         <f t="shared" si="0"/>
@@ -1257,7 +1257,7 @@
         <v>13</v>
       </c>
       <c r="G7" s="4" t="s">
-        <v>17</v>
+        <v>28</v>
       </c>
       <c r="H7" s="4"/>
       <c r="I7" s="4"/>
@@ -1281,7 +1281,7 @@
         <v>0.2361111111111111</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="E8" t="str">
         <f t="shared" si="0"/>
@@ -1291,7 +1291,7 @@
         <v>16</v>
       </c>
       <c r="G8" s="4" t="s">
-        <v>17</v>
+        <v>28</v>
       </c>
       <c r="H8" s="4"/>
       <c r="I8" s="4"/>
@@ -1315,14 +1315,14 @@
         <v>0.25</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="E9" t="str">
         <f t="shared" si="0"/>
         <v>test</v>
       </c>
       <c r="F9" s="4" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="G9" s="4"/>
       <c r="H9" s="4"/>
@@ -9232,7 +9232,7 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>8</v>
@@ -9240,7 +9240,7 @@
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B2" t="s">
         <v>14</v>
@@ -9248,18 +9248,18 @@
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B3" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B4" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
@@ -9275,15 +9275,15 @@
         <v>16</v>
       </c>
       <c r="B6" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
+        <v>24</v>
+      </c>
+      <c r="B7" t="s">
         <v>25</v>
-      </c>
-      <c r="B7" t="s">
-        <v>26</v>
       </c>
     </row>
   </sheetData>

</xml_diff>